<commit_message>
update files of job-to-machine
</commit_message>
<xml_diff>
--- a/AI Planning/Job Scheduling/Job To Machine/problemset/problemset.xlsx
+++ b/AI Planning/Job Scheduling/Job To Machine/problemset/problemset.xlsx
@@ -528,7 +528,7 @@
         <v>8</v>
       </c>
       <c r="F2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="G2" t="n">
         <v>9</v>
@@ -542,7 +542,7 @@
         <v>8</v>
       </c>
       <c r="J2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="K2" t="n">
         <v>9</v>
@@ -556,7 +556,7 @@
         <v>8</v>
       </c>
       <c r="N2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="O2" t="n">
         <v>9</v>
@@ -574,29 +574,29 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/mlf/delivery-10j-3m-1_10tr-uniformd-12c_mlf.xlsx</t>
+          <t>Job To Machine/problemset/solution/mlf/delivery-10j-3m-1_10tr-uniformd-13.0c_mlf.xlsx</t>
         </is>
       </c>
       <c r="E3" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="F3" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G3" t="n">
         <v>10</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/sjf/delivery-10j-3m-1_10tr-uniformd-12c_sjf.xlsx</t>
+          <t>Job To Machine/problemset/solution/sjf/delivery-10j-3m-1_10tr-uniformd-13.0c_sjf.xlsx</t>
         </is>
       </c>
       <c r="I3" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="J3" t="n">
         <v>2</v>
@@ -606,11 +606,11 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/ljf/delivery-10j-3m-1_10tr-uniformd-12c_ljf.xlsx</t>
+          <t>Job To Machine/problemset/solution/ljf/delivery-10j-3m-1_10tr-uniformd-13.0c_ljf.xlsx</t>
         </is>
       </c>
       <c r="M3" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="N3" t="n">
         <v>2</v>
@@ -688,15 +688,15 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/mlf/delivery-10j-3m-1_10tr-constantd-5c_mlf.xlsx</t>
+          <t>Job To Machine/problemset/solution/mlf/delivery-10j-3m-1_10tr-constantd-4.0c_mlf.xlsx</t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F5" t="n">
         <v>1</v>
@@ -706,11 +706,11 @@
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/sjf/delivery-10j-3m-1_10tr-constantd-5c_sjf.xlsx</t>
+          <t>Job To Machine/problemset/solution/sjf/delivery-10j-3m-1_10tr-constantd-4.0c_sjf.xlsx</t>
         </is>
       </c>
       <c r="I5" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J5" t="n">
         <v>1</v>
@@ -720,11 +720,11 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/ljf/delivery-10j-3m-1_10tr-constantd-5c_ljf.xlsx</t>
+          <t>Job To Machine/problemset/solution/ljf/delivery-10j-3m-1_10tr-constantd-4.0c_ljf.xlsx</t>
         </is>
       </c>
       <c r="M5" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="N5" t="n">
         <v>1</v>
@@ -745,49 +745,49 @@
         </is>
       </c>
       <c r="C6" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/mlf/delivery-10j-3m-1_10tr-normald-13c_mlf.xlsx</t>
+          <t>Job To Machine/problemset/solution/mlf/delivery-10j-3m-1_10tr-normald-11c_mlf.xlsx</t>
         </is>
       </c>
       <c r="E6" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="F6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G6" t="n">
         <v>8</v>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/sjf/delivery-10j-3m-1_10tr-normald-13c_sjf.xlsx</t>
+          <t>Job To Machine/problemset/solution/sjf/delivery-10j-3m-1_10tr-normald-11c_sjf.xlsx</t>
         </is>
       </c>
       <c r="I6" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="J6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K6" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/ljf/delivery-10j-3m-1_10tr-normald-13c_ljf.xlsx</t>
+          <t>Job To Machine/problemset/solution/ljf/delivery-10j-3m-1_10tr-normald-11c_ljf.xlsx</t>
         </is>
       </c>
       <c r="M6" t="n">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="N6" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O6" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="7">
@@ -802,46 +802,46 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>20</v>
+        <v>14</v>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/mlf/delivery-10j-3m-1_10tr-normald-20c_mlf.xlsx</t>
+          <t>Job To Machine/problemset/solution/mlf/delivery-10j-3m-1_10tr-normald-14.0c_mlf.xlsx</t>
         </is>
       </c>
       <c r="E7" t="n">
-        <v>19</v>
+        <v>12</v>
       </c>
       <c r="F7" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G7" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/sjf/delivery-10j-3m-1_10tr-normald-20c_sjf.xlsx</t>
+          <t>Job To Machine/problemset/solution/sjf/delivery-10j-3m-1_10tr-normald-14.0c_sjf.xlsx</t>
         </is>
       </c>
       <c r="I7" t="n">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="J7" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K7" t="n">
         <v>10</v>
       </c>
       <c r="L7" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/ljf/delivery-10j-3m-1_10tr-normald-20c_ljf.xlsx</t>
+          <t>Job To Machine/problemset/solution/ljf/delivery-10j-3m-1_10tr-normald-14.0c_ljf.xlsx</t>
         </is>
       </c>
       <c r="M7" t="n">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="N7" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="O7" t="n">
         <v>10</v>
@@ -873,7 +873,7 @@
         <v>1</v>
       </c>
       <c r="G8" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H8" t="inlineStr">
         <is>
@@ -887,7 +887,7 @@
         <v>1</v>
       </c>
       <c r="K8" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="L8" t="inlineStr">
         <is>
@@ -901,7 +901,7 @@
         <v>1</v>
       </c>
       <c r="O8" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="9">
@@ -920,7 +920,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/mlf/delivery-10j-3m-1_10tr-exponentiald-5c_mlf.xlsx</t>
+          <t>Job To Machine/problemset/solution/mlf/delivery-10j-3m-1_10tr-exponentiald-5.0c_mlf.xlsx</t>
         </is>
       </c>
       <c r="E9" t="n">
@@ -934,7 +934,7 @@
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/sjf/delivery-10j-3m-1_10tr-exponentiald-5c_sjf.xlsx</t>
+          <t>Job To Machine/problemset/solution/sjf/delivery-10j-3m-1_10tr-exponentiald-5.0c_sjf.xlsx</t>
         </is>
       </c>
       <c r="I9" t="n">
@@ -948,7 +948,7 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/ljf/delivery-10j-3m-1_10tr-exponentiald-5c_ljf.xlsx</t>
+          <t>Job To Machine/problemset/solution/ljf/delivery-10j-3m-1_10tr-exponentiald-5.0c_ljf.xlsx</t>
         </is>
       </c>
       <c r="M9" t="n">
@@ -973,49 +973,49 @@
         </is>
       </c>
       <c r="C10" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/mlf/delivery-10j-3m-1_10tr-lognormald-4c_mlf.xlsx</t>
+          <t>Job To Machine/problemset/solution/mlf/delivery-10j-3m-1_10tr-lognormald-8c_mlf.xlsx</t>
         </is>
       </c>
       <c r="E10" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="F10" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G10" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/sjf/delivery-10j-3m-1_10tr-lognormald-4c_sjf.xlsx</t>
+          <t>Job To Machine/problemset/solution/sjf/delivery-10j-3m-1_10tr-lognormald-8c_sjf.xlsx</t>
         </is>
       </c>
       <c r="I10" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="J10" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K10" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="L10" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/ljf/delivery-10j-3m-1_10tr-lognormald-4c_ljf.xlsx</t>
+          <t>Job To Machine/problemset/solution/ljf/delivery-10j-3m-1_10tr-lognormald-8c_ljf.xlsx</t>
         </is>
       </c>
       <c r="M10" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="N10" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O10" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
     </row>
     <row r="11">
@@ -1030,46 +1030,46 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/mlf/delivery-10j-3m-1_10tr-lognormald-7c_mlf.xlsx</t>
+          <t>Job To Machine/problemset/solution/mlf/delivery-10j-3m-1_10tr-lognormald-10.0c_mlf.xlsx</t>
         </is>
       </c>
       <c r="E11" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="F11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G11" t="n">
         <v>10</v>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/sjf/delivery-10j-3m-1_10tr-lognormald-7c_sjf.xlsx</t>
+          <t>Job To Machine/problemset/solution/sjf/delivery-10j-3m-1_10tr-lognormald-10.0c_sjf.xlsx</t>
         </is>
       </c>
       <c r="I11" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="J11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="K11" t="n">
         <v>10</v>
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/ljf/delivery-10j-3m-1_10tr-lognormald-7c_ljf.xlsx</t>
+          <t>Job To Machine/problemset/solution/ljf/delivery-10j-3m-1_10tr-lognormald-10.0c_ljf.xlsx</t>
         </is>
       </c>
       <c r="M11" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="N11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="O11" t="n">
         <v>10</v>
@@ -1087,49 +1087,49 @@
         </is>
       </c>
       <c r="C12" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/mlf/delivery-10j-3m-1_10tr-same_per_machined-10c_mlf.xlsx</t>
+          <t>Job To Machine/problemset/solution/mlf/delivery-10j-3m-1_10tr-same_per_machined-13c_mlf.xlsx</t>
         </is>
       </c>
       <c r="E12" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="F12" t="n">
         <v>5</v>
       </c>
       <c r="G12" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/sjf/delivery-10j-3m-1_10tr-same_per_machined-10c_sjf.xlsx</t>
+          <t>Job To Machine/problemset/solution/sjf/delivery-10j-3m-1_10tr-same_per_machined-13c_sjf.xlsx</t>
         </is>
       </c>
       <c r="I12" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="J12" t="n">
         <v>5</v>
       </c>
       <c r="K12" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="L12" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/ljf/delivery-10j-3m-1_10tr-same_per_machined-10c_ljf.xlsx</t>
+          <t>Job To Machine/problemset/solution/ljf/delivery-10j-3m-1_10tr-same_per_machined-13c_ljf.xlsx</t>
         </is>
       </c>
       <c r="M12" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="N12" t="n">
         <v>5</v>
       </c>
       <c r="O12" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="13">
@@ -1148,42 +1148,42 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/mlf/delivery-10j-3m-1_10tr-same_per_machined-15c_mlf.xlsx</t>
+          <t>Job To Machine/problemset/solution/mlf/delivery-10j-3m-1_10tr-same_per_machined-15.0c_mlf.xlsx</t>
         </is>
       </c>
       <c r="E13" t="n">
         <v>15</v>
       </c>
       <c r="F13" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="G13" t="n">
         <v>7</v>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/sjf/delivery-10j-3m-1_10tr-same_per_machined-15c_sjf.xlsx</t>
+          <t>Job To Machine/problemset/solution/sjf/delivery-10j-3m-1_10tr-same_per_machined-15.0c_sjf.xlsx</t>
         </is>
       </c>
       <c r="I13" t="n">
         <v>15</v>
       </c>
       <c r="J13" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="K13" t="n">
         <v>7</v>
       </c>
       <c r="L13" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/ljf/delivery-10j-3m-1_10tr-same_per_machined-15c_ljf.xlsx</t>
+          <t>Job To Machine/problemset/solution/ljf/delivery-10j-3m-1_10tr-same_per_machined-15.0c_ljf.xlsx</t>
         </is>
       </c>
       <c r="M13" t="n">
         <v>15</v>
       </c>
       <c r="N13" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="O13" t="n">
         <v>7</v>
@@ -1201,46 +1201,46 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/mlf/delivery-10j-3m-1_10tr-same_per_jobd-12c_mlf.xlsx</t>
+          <t>Job To Machine/problemset/solution/mlf/delivery-10j-3m-1_10tr-same_per_jobd-20c_mlf.xlsx</t>
         </is>
       </c>
       <c r="E14" t="n">
-        <v>12</v>
+        <v>19</v>
       </c>
       <c r="F14" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="G14" t="n">
         <v>9</v>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/sjf/delivery-10j-3m-1_10tr-same_per_jobd-12c_sjf.xlsx</t>
+          <t>Job To Machine/problemset/solution/sjf/delivery-10j-3m-1_10tr-same_per_jobd-20c_sjf.xlsx</t>
         </is>
       </c>
       <c r="I14" t="n">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="J14" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="K14" t="n">
         <v>9</v>
       </c>
       <c r="L14" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/ljf/delivery-10j-3m-1_10tr-same_per_jobd-12c_ljf.xlsx</t>
+          <t>Job To Machine/problemset/solution/ljf/delivery-10j-3m-1_10tr-same_per_jobd-20c_ljf.xlsx</t>
         </is>
       </c>
       <c r="M14" t="n">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="N14" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="O14" t="n">
         <v>9</v>
@@ -1258,49 +1258,49 @@
         </is>
       </c>
       <c r="C15" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/mlf/delivery-10j-3m-1_10tr-same_per_jobd-18c_mlf.xlsx</t>
+          <t>Job To Machine/problemset/solution/mlf/delivery-10j-3m-1_10tr-same_per_jobd-20.0c_mlf.xlsx</t>
         </is>
       </c>
       <c r="E15" t="n">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="F15" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="G15" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/sjf/delivery-10j-3m-1_10tr-same_per_jobd-18c_sjf.xlsx</t>
+          <t>Job To Machine/problemset/solution/sjf/delivery-10j-3m-1_10tr-same_per_jobd-20.0c_sjf.xlsx</t>
         </is>
       </c>
       <c r="I15" t="n">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="J15" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="K15" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="L15" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/ljf/delivery-10j-3m-1_10tr-same_per_jobd-18c_ljf.xlsx</t>
+          <t>Job To Machine/problemset/solution/ljf/delivery-10j-3m-1_10tr-same_per_jobd-20.0c_ljf.xlsx</t>
         </is>
       </c>
       <c r="M15" t="n">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="N15" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="O15" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="16">
@@ -1315,49 +1315,49 @@
         </is>
       </c>
       <c r="C16" t="n">
-        <v>123</v>
+        <v>99</v>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/mlf/banco-30j-4m-5_60tr-uniformd-123c_mlf.xlsx</t>
+          <t>Job To Machine/problemset/solution/mlf/banco-30j-4m-5_60tr-uniformd-99c_mlf.xlsx</t>
         </is>
       </c>
       <c r="E16" t="n">
-        <v>121</v>
+        <v>98</v>
       </c>
       <c r="F16" t="n">
         <v>16</v>
       </c>
       <c r="G16" t="n">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/sjf/banco-30j-4m-5_60tr-uniformd-123c_sjf.xlsx</t>
+          <t>Job To Machine/problemset/solution/sjf/banco-30j-4m-5_60tr-uniformd-99c_sjf.xlsx</t>
         </is>
       </c>
       <c r="I16" t="n">
-        <v>121</v>
+        <v>94</v>
       </c>
       <c r="J16" t="n">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="K16" t="n">
         <v>27</v>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/ljf/banco-30j-4m-5_60tr-uniformd-123c_ljf.xlsx</t>
+          <t>Job To Machine/problemset/solution/ljf/banco-30j-4m-5_60tr-uniformd-99c_ljf.xlsx</t>
         </is>
       </c>
       <c r="M16" t="n">
-        <v>121</v>
+        <v>99</v>
       </c>
       <c r="N16" t="n">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="O16" t="n">
-        <v>27</v>
+        <v>26</v>
       </c>
     </row>
     <row r="17">
@@ -1372,46 +1372,46 @@
         </is>
       </c>
       <c r="C17" t="n">
-        <v>165</v>
+        <v>156</v>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/mlf/banco-30j-4m-5_60tr-uniformd-165c_mlf.xlsx</t>
+          <t>Job To Machine/problemset/solution/mlf/banco-30j-4m-5_60tr-uniformd-156.0c_mlf.xlsx</t>
         </is>
       </c>
       <c r="E17" t="n">
-        <v>156</v>
+        <v>139</v>
       </c>
       <c r="F17" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="G17" t="n">
         <v>30</v>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/sjf/banco-30j-4m-5_60tr-uniformd-165c_sjf.xlsx</t>
+          <t>Job To Machine/problemset/solution/sjf/banco-30j-4m-5_60tr-uniformd-156.0c_sjf.xlsx</t>
         </is>
       </c>
       <c r="I17" t="n">
-        <v>156</v>
+        <v>139</v>
       </c>
       <c r="J17" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="K17" t="n">
         <v>30</v>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/ljf/banco-30j-4m-5_60tr-uniformd-165c_ljf.xlsx</t>
+          <t>Job To Machine/problemset/solution/ljf/banco-30j-4m-5_60tr-uniformd-156.0c_ljf.xlsx</t>
         </is>
       </c>
       <c r="M17" t="n">
-        <v>156</v>
+        <v>139</v>
       </c>
       <c r="N17" t="n">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="O17" t="n">
         <v>30</v>
@@ -1486,49 +1486,49 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>50</v>
+        <v>38</v>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/mlf/banco-30j-4m-5_60tr-constantd-50c_mlf.xlsx</t>
+          <t>Job To Machine/problemset/solution/mlf/banco-30j-4m-5_60tr-constantd-38.0c_mlf.xlsx</t>
         </is>
       </c>
       <c r="E19" t="n">
-        <v>50</v>
+        <v>35</v>
       </c>
       <c r="F19" t="n">
         <v>5</v>
       </c>
       <c r="G19" t="n">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/sjf/banco-30j-4m-5_60tr-constantd-50c_sjf.xlsx</t>
+          <t>Job To Machine/problemset/solution/sjf/banco-30j-4m-5_60tr-constantd-38.0c_sjf.xlsx</t>
         </is>
       </c>
       <c r="I19" t="n">
-        <v>50</v>
+        <v>35</v>
       </c>
       <c r="J19" t="n">
         <v>5</v>
       </c>
       <c r="K19" t="n">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/ljf/banco-30j-4m-5_60tr-constantd-50c_ljf.xlsx</t>
+          <t>Job To Machine/problemset/solution/ljf/banco-30j-4m-5_60tr-constantd-38.0c_ljf.xlsx</t>
         </is>
       </c>
       <c r="M19" t="n">
-        <v>50</v>
+        <v>35</v>
       </c>
       <c r="N19" t="n">
         <v>5</v>
       </c>
       <c r="O19" t="n">
-        <v>30</v>
+        <v>28</v>
       </c>
     </row>
     <row r="20">
@@ -1543,46 +1543,46 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>120</v>
+        <v>138</v>
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/mlf/banco-30j-4m-5_60tr-normald-120c_mlf.xlsx</t>
+          <t>Job To Machine/problemset/solution/mlf/banco-30j-4m-5_60tr-normald-138c_mlf.xlsx</t>
         </is>
       </c>
       <c r="E20" t="n">
-        <v>118</v>
+        <v>138</v>
       </c>
       <c r="F20" t="n">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="G20" t="n">
         <v>28</v>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/sjf/banco-30j-4m-5_60tr-normald-120c_sjf.xlsx</t>
+          <t>Job To Machine/problemset/solution/sjf/banco-30j-4m-5_60tr-normald-138c_sjf.xlsx</t>
         </is>
       </c>
       <c r="I20" t="n">
-        <v>118</v>
+        <v>137</v>
       </c>
       <c r="J20" t="n">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="K20" t="n">
         <v>28</v>
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/ljf/banco-30j-4m-5_60tr-normald-120c_ljf.xlsx</t>
+          <t>Job To Machine/problemset/solution/ljf/banco-30j-4m-5_60tr-normald-138c_ljf.xlsx</t>
         </is>
       </c>
       <c r="M20" t="n">
-        <v>118</v>
+        <v>138</v>
       </c>
       <c r="N20" t="n">
-        <v>15</v>
+        <v>19</v>
       </c>
       <c r="O20" t="n">
         <v>28</v>
@@ -1600,46 +1600,46 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>161</v>
+        <v>178</v>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/mlf/banco-30j-4m-5_60tr-normald-161c_mlf.xlsx</t>
+          <t>Job To Machine/problemset/solution/mlf/banco-30j-4m-5_60tr-normald-178.0c_mlf.xlsx</t>
         </is>
       </c>
       <c r="E21" t="n">
-        <v>143</v>
+        <v>169</v>
       </c>
       <c r="F21" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="G21" t="n">
         <v>30</v>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/sjf/banco-30j-4m-5_60tr-normald-161c_sjf.xlsx</t>
+          <t>Job To Machine/problemset/solution/sjf/banco-30j-4m-5_60tr-normald-178.0c_sjf.xlsx</t>
         </is>
       </c>
       <c r="I21" t="n">
-        <v>143</v>
+        <v>170</v>
       </c>
       <c r="J21" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="K21" t="n">
         <v>30</v>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/ljf/banco-30j-4m-5_60tr-normald-161c_ljf.xlsx</t>
+          <t>Job To Machine/problemset/solution/ljf/banco-30j-4m-5_60tr-normald-178.0c_ljf.xlsx</t>
         </is>
       </c>
       <c r="M21" t="n">
-        <v>143</v>
+        <v>177</v>
       </c>
       <c r="N21" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="O21" t="n">
         <v>30</v>
@@ -1657,49 +1657,49 @@
         </is>
       </c>
       <c r="C22" t="n">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/mlf/banco-30j-4m-5_60tr-exponentiald-55c_mlf.xlsx</t>
+          <t>Job To Machine/problemset/solution/mlf/banco-30j-4m-5_60tr-exponentiald-54c_mlf.xlsx</t>
         </is>
       </c>
       <c r="E22" t="n">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="F22" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="G22" t="n">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/sjf/banco-30j-4m-5_60tr-exponentiald-55c_sjf.xlsx</t>
+          <t>Job To Machine/problemset/solution/sjf/banco-30j-4m-5_60tr-exponentiald-54c_sjf.xlsx</t>
         </is>
       </c>
       <c r="I22" t="n">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="J22" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="K22" t="n">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/ljf/banco-30j-4m-5_60tr-exponentiald-55c_ljf.xlsx</t>
+          <t>Job To Machine/problemset/solution/ljf/banco-30j-4m-5_60tr-exponentiald-54c_ljf.xlsx</t>
         </is>
       </c>
       <c r="M22" t="n">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="N22" t="n">
         <v>8</v>
       </c>
       <c r="O22" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="23">
@@ -1714,11 +1714,11 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/mlf/banco-30j-4m-5_60tr-exponentiald-74c_mlf.xlsx</t>
+          <t>Job To Machine/problemset/solution/mlf/banco-30j-4m-5_60tr-exponentiald-71.0c_mlf.xlsx</t>
         </is>
       </c>
       <c r="E23" t="n">
@@ -1732,7 +1732,7 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/sjf/banco-30j-4m-5_60tr-exponentiald-74c_sjf.xlsx</t>
+          <t>Job To Machine/problemset/solution/sjf/banco-30j-4m-5_60tr-exponentiald-71.0c_sjf.xlsx</t>
         </is>
       </c>
       <c r="I23" t="n">
@@ -1746,7 +1746,7 @@
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/ljf/banco-30j-4m-5_60tr-exponentiald-74c_ljf.xlsx</t>
+          <t>Job To Machine/problemset/solution/ljf/banco-30j-4m-5_60tr-exponentiald-71.0c_ljf.xlsx</t>
         </is>
       </c>
       <c r="M23" t="n">
@@ -1771,49 +1771,49 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>104</v>
+        <v>99</v>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/mlf/banco-30j-4m-5_60tr-lognormald-104c_mlf.xlsx</t>
+          <t>Job To Machine/problemset/solution/mlf/banco-30j-4m-5_60tr-lognormald-99c_mlf.xlsx</t>
         </is>
       </c>
       <c r="E24" t="n">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="F24" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="G24" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/sjf/banco-30j-4m-5_60tr-lognormald-104c_sjf.xlsx</t>
+          <t>Job To Machine/problemset/solution/sjf/banco-30j-4m-5_60tr-lognormald-99c_sjf.xlsx</t>
         </is>
       </c>
       <c r="I24" t="n">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="J24" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="K24" t="n">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/ljf/banco-30j-4m-5_60tr-lognormald-104c_ljf.xlsx</t>
+          <t>Job To Machine/problemset/solution/ljf/banco-30j-4m-5_60tr-lognormald-99c_ljf.xlsx</t>
         </is>
       </c>
       <c r="M24" t="n">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="N24" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="O24" t="n">
-        <v>26</v>
+        <v>28</v>
       </c>
     </row>
     <row r="25">
@@ -1828,46 +1828,46 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>138</v>
+        <v>125</v>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/mlf/banco-30j-4m-5_60tr-lognormald-138c_mlf.xlsx</t>
+          <t>Job To Machine/problemset/solution/mlf/banco-30j-4m-5_60tr-lognormald-125.0c_mlf.xlsx</t>
         </is>
       </c>
       <c r="E25" t="n">
-        <v>134</v>
+        <v>119</v>
       </c>
       <c r="F25" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="G25" t="n">
         <v>30</v>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/sjf/banco-30j-4m-5_60tr-lognormald-138c_sjf.xlsx</t>
+          <t>Job To Machine/problemset/solution/sjf/banco-30j-4m-5_60tr-lognormald-125.0c_sjf.xlsx</t>
         </is>
       </c>
       <c r="I25" t="n">
-        <v>134</v>
+        <v>115</v>
       </c>
       <c r="J25" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="K25" t="n">
         <v>30</v>
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/ljf/banco-30j-4m-5_60tr-lognormald-138c_ljf.xlsx</t>
+          <t>Job To Machine/problemset/solution/ljf/banco-30j-4m-5_60tr-lognormald-125.0c_ljf.xlsx</t>
         </is>
       </c>
       <c r="M25" t="n">
-        <v>134</v>
+        <v>124</v>
       </c>
       <c r="N25" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="O25" t="n">
         <v>30</v>
@@ -1885,49 +1885,49 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>172</v>
+        <v>37</v>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/mlf/banco-30j-4m-5_60tr-same_per_machined-172c_mlf.xlsx</t>
+          <t>Job To Machine/problemset/solution/mlf/banco-30j-4m-5_60tr-same_per_machined-37c_mlf.xlsx</t>
         </is>
       </c>
       <c r="E26" t="n">
-        <v>161</v>
+        <v>35</v>
       </c>
       <c r="F26" t="n">
-        <v>33</v>
+        <v>11</v>
       </c>
       <c r="G26" t="n">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/sjf/banco-30j-4m-5_60tr-same_per_machined-172c_sjf.xlsx</t>
+          <t>Job To Machine/problemset/solution/sjf/banco-30j-4m-5_60tr-same_per_machined-37c_sjf.xlsx</t>
         </is>
       </c>
       <c r="I26" t="n">
-        <v>161</v>
+        <v>35</v>
       </c>
       <c r="J26" t="n">
-        <v>33</v>
+        <v>11</v>
       </c>
       <c r="K26" t="n">
-        <v>17</v>
+        <v>10</v>
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/ljf/banco-30j-4m-5_60tr-same_per_machined-172c_ljf.xlsx</t>
+          <t>Job To Machine/problemset/solution/ljf/banco-30j-4m-5_60tr-same_per_machined-37c_ljf.xlsx</t>
         </is>
       </c>
       <c r="M26" t="n">
-        <v>161</v>
+        <v>35</v>
       </c>
       <c r="N26" t="n">
-        <v>33</v>
+        <v>11</v>
       </c>
       <c r="O26" t="n">
-        <v>17</v>
+        <v>10</v>
       </c>
     </row>
     <row r="27">
@@ -1942,49 +1942,49 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>230</v>
+        <v>106</v>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/mlf/banco-30j-4m-5_60tr-same_per_machined-230c_mlf.xlsx</t>
+          <t>Job To Machine/problemset/solution/mlf/banco-30j-4m-5_60tr-same_per_machined-106.0c_mlf.xlsx</t>
         </is>
       </c>
       <c r="E27" t="n">
-        <v>230</v>
+        <v>105</v>
       </c>
       <c r="F27" t="n">
-        <v>34</v>
+        <v>10</v>
       </c>
       <c r="G27" t="n">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/sjf/banco-30j-4m-5_60tr-same_per_machined-230c_sjf.xlsx</t>
+          <t>Job To Machine/problemset/solution/sjf/banco-30j-4m-5_60tr-same_per_machined-106.0c_sjf.xlsx</t>
         </is>
       </c>
       <c r="I27" t="n">
-        <v>230</v>
+        <v>105</v>
       </c>
       <c r="J27" t="n">
-        <v>34</v>
+        <v>10</v>
       </c>
       <c r="K27" t="n">
-        <v>25</v>
+        <v>30</v>
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/ljf/banco-30j-4m-5_60tr-same_per_machined-230c_ljf.xlsx</t>
+          <t>Job To Machine/problemset/solution/ljf/banco-30j-4m-5_60tr-same_per_machined-106.0c_ljf.xlsx</t>
         </is>
       </c>
       <c r="M27" t="n">
-        <v>230</v>
+        <v>105</v>
       </c>
       <c r="N27" t="n">
-        <v>34</v>
+        <v>10</v>
       </c>
       <c r="O27" t="n">
-        <v>25</v>
+        <v>30</v>
       </c>
     </row>
     <row r="28">
@@ -1999,46 +1999,46 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>250</v>
+        <v>203</v>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/mlf/banco-30j-4m-5_60tr-same_per_jobd-250c_mlf.xlsx</t>
+          <t>Job To Machine/problemset/solution/mlf/banco-30j-4m-5_60tr-same_per_jobd-203c_mlf.xlsx</t>
         </is>
       </c>
       <c r="E28" t="n">
-        <v>250</v>
+        <v>202</v>
       </c>
       <c r="F28" t="n">
-        <v>33</v>
+        <v>26</v>
       </c>
       <c r="G28" t="n">
         <v>29</v>
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/sjf/banco-30j-4m-5_60tr-same_per_jobd-250c_sjf.xlsx</t>
+          <t>Job To Machine/problemset/solution/sjf/banco-30j-4m-5_60tr-same_per_jobd-203c_sjf.xlsx</t>
         </is>
       </c>
       <c r="I28" t="n">
-        <v>250</v>
+        <v>196</v>
       </c>
       <c r="J28" t="n">
-        <v>33</v>
+        <v>26</v>
       </c>
       <c r="K28" t="n">
         <v>29</v>
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/ljf/banco-30j-4m-5_60tr-same_per_jobd-250c_ljf.xlsx</t>
+          <t>Job To Machine/problemset/solution/ljf/banco-30j-4m-5_60tr-same_per_jobd-203c_ljf.xlsx</t>
         </is>
       </c>
       <c r="M28" t="n">
-        <v>250</v>
+        <v>196</v>
       </c>
       <c r="N28" t="n">
-        <v>33</v>
+        <v>26</v>
       </c>
       <c r="O28" t="n">
         <v>29</v>
@@ -2056,49 +2056,49 @@
         </is>
       </c>
       <c r="C29" t="n">
-        <v>334</v>
+        <v>204</v>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/mlf/banco-30j-4m-5_60tr-same_per_jobd-334c_mlf.xlsx</t>
+          <t>Job To Machine/problemset/solution/mlf/banco-30j-4m-5_60tr-same_per_jobd-204.0c_mlf.xlsx</t>
         </is>
       </c>
       <c r="E29" t="n">
-        <v>334</v>
+        <v>202</v>
       </c>
       <c r="F29" t="n">
-        <v>33</v>
+        <v>26</v>
       </c>
       <c r="G29" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/sjf/banco-30j-4m-5_60tr-same_per_jobd-334c_sjf.xlsx</t>
+          <t>Job To Machine/problemset/solution/sjf/banco-30j-4m-5_60tr-same_per_jobd-204.0c_sjf.xlsx</t>
         </is>
       </c>
       <c r="I29" t="n">
-        <v>334</v>
+        <v>196</v>
       </c>
       <c r="J29" t="n">
-        <v>33</v>
+        <v>26</v>
       </c>
       <c r="K29" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/ljf/banco-30j-4m-5_60tr-same_per_jobd-334c_ljf.xlsx</t>
+          <t>Job To Machine/problemset/solution/ljf/banco-30j-4m-5_60tr-same_per_jobd-204.0c_ljf.xlsx</t>
         </is>
       </c>
       <c r="M29" t="n">
-        <v>334</v>
+        <v>196</v>
       </c>
       <c r="N29" t="n">
-        <v>33</v>
+        <v>26</v>
       </c>
       <c r="O29" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="30">
@@ -2113,49 +2113,49 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>854</v>
+        <v>837</v>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/mlf/reparacion-150j-10m-30_300tr-uniformd-854c_mlf.xlsx</t>
+          <t>Job To Machine/problemset/solution/mlf/reparacion-150j-10m-30_300tr-uniformd-837c_mlf.xlsx</t>
         </is>
       </c>
       <c r="E30" t="n">
-        <v>854</v>
+        <v>830</v>
       </c>
       <c r="F30" t="n">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="G30" t="n">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/sjf/reparacion-150j-10m-30_300tr-uniformd-854c_sjf.xlsx</t>
+          <t>Job To Machine/problemset/solution/sjf/reparacion-150j-10m-30_300tr-uniformd-837c_sjf.xlsx</t>
         </is>
       </c>
       <c r="I30" t="n">
-        <v>854</v>
+        <v>820</v>
       </c>
       <c r="J30" t="n">
-        <v>60</v>
+        <v>54</v>
       </c>
       <c r="K30" t="n">
-        <v>138</v>
+        <v>142</v>
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/ljf/reparacion-150j-10m-30_300tr-uniformd-854c_ljf.xlsx</t>
+          <t>Job To Machine/problemset/solution/ljf/reparacion-150j-10m-30_300tr-uniformd-837c_ljf.xlsx</t>
         </is>
       </c>
       <c r="M30" t="n">
-        <v>854</v>
+        <v>837</v>
       </c>
       <c r="N30" t="n">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="O30" t="n">
-        <v>138</v>
+        <v>135</v>
       </c>
     </row>
     <row r="31">
@@ -2170,49 +2170,49 @@
         </is>
       </c>
       <c r="C31" t="n">
-        <v>949</v>
+        <v>1511</v>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/mlf/reparacion-150j-10m-30_300tr-uniformd-949c_mlf.xlsx</t>
+          <t>Job To Machine/problemset/solution/mlf/reparacion-150j-10m-30_300tr-uniformd-1511.0c_mlf.xlsx</t>
         </is>
       </c>
       <c r="E31" t="n">
-        <v>944</v>
+        <v>1335</v>
       </c>
       <c r="F31" t="n">
-        <v>61</v>
+        <v>55</v>
       </c>
       <c r="G31" t="n">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/sjf/reparacion-150j-10m-30_300tr-uniformd-949c_sjf.xlsx</t>
+          <t>Job To Machine/problemset/solution/sjf/reparacion-150j-10m-30_300tr-uniformd-1511.0c_sjf.xlsx</t>
         </is>
       </c>
       <c r="I31" t="n">
-        <v>944</v>
+        <v>1335</v>
       </c>
       <c r="J31" t="n">
-        <v>61</v>
+        <v>55</v>
       </c>
       <c r="K31" t="n">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/ljf/reparacion-150j-10m-30_300tr-uniformd-949c_ljf.xlsx</t>
+          <t>Job To Machine/problemset/solution/ljf/reparacion-150j-10m-30_300tr-uniformd-1511.0c_ljf.xlsx</t>
         </is>
       </c>
       <c r="M31" t="n">
-        <v>944</v>
+        <v>1335</v>
       </c>
       <c r="N31" t="n">
-        <v>61</v>
+        <v>55</v>
       </c>
       <c r="O31" t="n">
-        <v>148</v>
+        <v>150</v>
       </c>
     </row>
     <row r="32">
@@ -2284,15 +2284,15 @@
         </is>
       </c>
       <c r="C33" t="n">
-        <v>500</v>
+        <v>450</v>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/mlf/reparacion-150j-10m-30_300tr-constantd-500c_mlf.xlsx</t>
+          <t>Job To Machine/problemset/solution/mlf/reparacion-150j-10m-30_300tr-constantd-450.0c_mlf.xlsx</t>
         </is>
       </c>
       <c r="E33" t="n">
-        <v>480</v>
+        <v>450</v>
       </c>
       <c r="F33" t="n">
         <v>30</v>
@@ -2302,11 +2302,11 @@
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/sjf/reparacion-150j-10m-30_300tr-constantd-500c_sjf.xlsx</t>
+          <t>Job To Machine/problemset/solution/sjf/reparacion-150j-10m-30_300tr-constantd-450.0c_sjf.xlsx</t>
         </is>
       </c>
       <c r="I33" t="n">
-        <v>480</v>
+        <v>450</v>
       </c>
       <c r="J33" t="n">
         <v>30</v>
@@ -2316,11 +2316,11 @@
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/ljf/reparacion-150j-10m-30_300tr-constantd-500c_ljf.xlsx</t>
+          <t>Job To Machine/problemset/solution/ljf/reparacion-150j-10m-30_300tr-constantd-450.0c_ljf.xlsx</t>
         </is>
       </c>
       <c r="M33" t="n">
-        <v>480</v>
+        <v>450</v>
       </c>
       <c r="N33" t="n">
         <v>30</v>
@@ -2341,49 +2341,49 @@
         </is>
       </c>
       <c r="C34" t="n">
-        <v>987</v>
+        <v>970</v>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/mlf/reparacion-150j-10m-30_300tr-normald-987c_mlf.xlsx</t>
+          <t>Job To Machine/problemset/solution/mlf/reparacion-150j-10m-30_300tr-normald-970c_mlf.xlsx</t>
         </is>
       </c>
       <c r="E34" t="n">
-        <v>982</v>
+        <v>969</v>
       </c>
       <c r="F34" t="n">
         <v>69</v>
       </c>
       <c r="G34" t="n">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/sjf/reparacion-150j-10m-30_300tr-normald-987c_sjf.xlsx</t>
+          <t>Job To Machine/problemset/solution/sjf/reparacion-150j-10m-30_300tr-normald-970c_sjf.xlsx</t>
         </is>
       </c>
       <c r="I34" t="n">
-        <v>982</v>
+        <v>963</v>
       </c>
       <c r="J34" t="n">
-        <v>69</v>
+        <v>63</v>
       </c>
       <c r="K34" t="n">
-        <v>137</v>
+        <v>145</v>
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/ljf/reparacion-150j-10m-30_300tr-normald-987c_ljf.xlsx</t>
+          <t>Job To Machine/problemset/solution/ljf/reparacion-150j-10m-30_300tr-normald-970c_ljf.xlsx</t>
         </is>
       </c>
       <c r="M34" t="n">
-        <v>982</v>
+        <v>970</v>
       </c>
       <c r="N34" t="n">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="O34" t="n">
-        <v>137</v>
+        <v>142</v>
       </c>
     </row>
     <row r="35">
@@ -2398,46 +2398,46 @@
         </is>
       </c>
       <c r="C35" t="n">
-        <v>1096</v>
+        <v>1693</v>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/mlf/reparacion-150j-10m-30_300tr-normald-1096c_mlf.xlsx</t>
+          <t>Job To Machine/problemset/solution/mlf/reparacion-150j-10m-30_300tr-normald-1693.0c_mlf.xlsx</t>
         </is>
       </c>
       <c r="E35" t="n">
-        <v>1096</v>
+        <v>1255</v>
       </c>
       <c r="F35" t="n">
-        <v>70</v>
+        <v>64</v>
       </c>
       <c r="G35" t="n">
         <v>150</v>
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/sjf/reparacion-150j-10m-30_300tr-normald-1096c_sjf.xlsx</t>
+          <t>Job To Machine/problemset/solution/sjf/reparacion-150j-10m-30_300tr-normald-1693.0c_sjf.xlsx</t>
         </is>
       </c>
       <c r="I35" t="n">
-        <v>1096</v>
+        <v>1255</v>
       </c>
       <c r="J35" t="n">
-        <v>70</v>
+        <v>64</v>
       </c>
       <c r="K35" t="n">
         <v>150</v>
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/ljf/reparacion-150j-10m-30_300tr-normald-1096c_ljf.xlsx</t>
+          <t>Job To Machine/problemset/solution/ljf/reparacion-150j-10m-30_300tr-normald-1693.0c_ljf.xlsx</t>
         </is>
       </c>
       <c r="M35" t="n">
-        <v>1096</v>
+        <v>1255</v>
       </c>
       <c r="N35" t="n">
-        <v>70</v>
+        <v>64</v>
       </c>
       <c r="O35" t="n">
         <v>150</v>
@@ -2455,29 +2455,29 @@
         </is>
       </c>
       <c r="C36" t="n">
-        <v>523</v>
+        <v>526</v>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/mlf/reparacion-150j-10m-30_300tr-exponentiald-523c_mlf.xlsx</t>
+          <t>Job To Machine/problemset/solution/mlf/reparacion-150j-10m-30_300tr-exponentiald-526c_mlf.xlsx</t>
         </is>
       </c>
       <c r="E36" t="n">
-        <v>518</v>
+        <v>525</v>
       </c>
       <c r="F36" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="G36" t="n">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/sjf/reparacion-150j-10m-30_300tr-exponentiald-523c_sjf.xlsx</t>
+          <t>Job To Machine/problemset/solution/sjf/reparacion-150j-10m-30_300tr-exponentiald-526c_sjf.xlsx</t>
         </is>
       </c>
       <c r="I36" t="n">
-        <v>518</v>
+        <v>521</v>
       </c>
       <c r="J36" t="n">
         <v>35</v>
@@ -2487,17 +2487,17 @@
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/ljf/reparacion-150j-10m-30_300tr-exponentiald-523c_ljf.xlsx</t>
+          <t>Job To Machine/problemset/solution/ljf/reparacion-150j-10m-30_300tr-exponentiald-526c_ljf.xlsx</t>
         </is>
       </c>
       <c r="M36" t="n">
-        <v>518</v>
+        <v>525</v>
       </c>
       <c r="N36" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="O36" t="n">
-        <v>142</v>
+        <v>139</v>
       </c>
     </row>
     <row r="37">
@@ -2512,15 +2512,15 @@
         </is>
       </c>
       <c r="C37" t="n">
-        <v>582</v>
+        <v>710</v>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/mlf/reparacion-150j-10m-30_300tr-exponentiald-582c_mlf.xlsx</t>
+          <t>Job To Machine/problemset/solution/mlf/reparacion-150j-10m-30_300tr-exponentiald-710.0c_mlf.xlsx</t>
         </is>
       </c>
       <c r="E37" t="n">
-        <v>582</v>
+        <v>699</v>
       </c>
       <c r="F37" t="n">
         <v>35</v>
@@ -2530,11 +2530,11 @@
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/sjf/reparacion-150j-10m-30_300tr-exponentiald-582c_sjf.xlsx</t>
+          <t>Job To Machine/problemset/solution/sjf/reparacion-150j-10m-30_300tr-exponentiald-710.0c_sjf.xlsx</t>
         </is>
       </c>
       <c r="I37" t="n">
-        <v>582</v>
+        <v>677</v>
       </c>
       <c r="J37" t="n">
         <v>35</v>
@@ -2544,11 +2544,11 @@
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/ljf/reparacion-150j-10m-30_300tr-exponentiald-582c_ljf.xlsx</t>
+          <t>Job To Machine/problemset/solution/ljf/reparacion-150j-10m-30_300tr-exponentiald-710.0c_ljf.xlsx</t>
         </is>
       </c>
       <c r="M37" t="n">
-        <v>582</v>
+        <v>692</v>
       </c>
       <c r="N37" t="n">
         <v>35</v>
@@ -2569,46 +2569,46 @@
         </is>
       </c>
       <c r="C38" t="n">
-        <v>1030</v>
+        <v>974</v>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/mlf/reparacion-150j-10m-30_300tr-lognormald-1030c_mlf.xlsx</t>
+          <t>Job To Machine/problemset/solution/mlf/reparacion-150j-10m-30_300tr-lognormald-974c_mlf.xlsx</t>
         </is>
       </c>
       <c r="E38" t="n">
-        <v>1030</v>
+        <v>973</v>
       </c>
       <c r="F38" t="n">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="G38" t="n">
-        <v>143</v>
+        <v>140</v>
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/sjf/reparacion-150j-10m-30_300tr-lognormald-1030c_sjf.xlsx</t>
+          <t>Job To Machine/problemset/solution/sjf/reparacion-150j-10m-30_300tr-lognormald-974c_sjf.xlsx</t>
         </is>
       </c>
       <c r="I38" t="n">
-        <v>1030</v>
+        <v>969</v>
       </c>
       <c r="J38" t="n">
-        <v>70</v>
+        <v>64</v>
       </c>
       <c r="K38" t="n">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/ljf/reparacion-150j-10m-30_300tr-lognormald-1030c_ljf.xlsx</t>
+          <t>Job To Machine/problemset/solution/ljf/reparacion-150j-10m-30_300tr-lognormald-974c_ljf.xlsx</t>
         </is>
       </c>
       <c r="M38" t="n">
-        <v>1030</v>
+        <v>972</v>
       </c>
       <c r="N38" t="n">
-        <v>70</v>
+        <v>66</v>
       </c>
       <c r="O38" t="n">
         <v>143</v>
@@ -2626,46 +2626,46 @@
         </is>
       </c>
       <c r="C39" t="n">
-        <v>1145</v>
+        <v>1290</v>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/mlf/reparacion-150j-10m-30_300tr-lognormald-1145c_mlf.xlsx</t>
+          <t>Job To Machine/problemset/solution/mlf/reparacion-150j-10m-30_300tr-lognormald-1290.0c_mlf.xlsx</t>
         </is>
       </c>
       <c r="E39" t="n">
-        <v>1142</v>
+        <v>1268</v>
       </c>
       <c r="F39" t="n">
-        <v>70</v>
+        <v>64</v>
       </c>
       <c r="G39" t="n">
         <v>150</v>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/sjf/reparacion-150j-10m-30_300tr-lognormald-1145c_sjf.xlsx</t>
+          <t>Job To Machine/problemset/solution/sjf/reparacion-150j-10m-30_300tr-lognormald-1290.0c_sjf.xlsx</t>
         </is>
       </c>
       <c r="I39" t="n">
-        <v>1142</v>
+        <v>1268</v>
       </c>
       <c r="J39" t="n">
-        <v>70</v>
+        <v>64</v>
       </c>
       <c r="K39" t="n">
         <v>150</v>
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/ljf/reparacion-150j-10m-30_300tr-lognormald-1145c_ljf.xlsx</t>
+          <t>Job To Machine/problemset/solution/ljf/reparacion-150j-10m-30_300tr-lognormald-1290.0c_ljf.xlsx</t>
         </is>
       </c>
       <c r="M39" t="n">
-        <v>1142</v>
+        <v>1268</v>
       </c>
       <c r="N39" t="n">
-        <v>70</v>
+        <v>64</v>
       </c>
       <c r="O39" t="n">
         <v>150</v>
@@ -2683,49 +2683,49 @@
         </is>
       </c>
       <c r="C40" t="n">
-        <v>780</v>
+        <v>705</v>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/mlf/reparacion-150j-10m-30_300tr-same_per_machined-780c_mlf.xlsx</t>
+          <t>Job To Machine/problemset/solution/mlf/reparacion-150j-10m-30_300tr-same_per_machined-705c_mlf.xlsx</t>
         </is>
       </c>
       <c r="E40" t="n">
-        <v>780</v>
+        <v>705</v>
       </c>
       <c r="F40" t="n">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="G40" t="n">
-        <v>63</v>
+        <v>52</v>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/sjf/reparacion-150j-10m-30_300tr-same_per_machined-780c_sjf.xlsx</t>
+          <t>Job To Machine/problemset/solution/sjf/reparacion-150j-10m-30_300tr-same_per_machined-705c_sjf.xlsx</t>
         </is>
       </c>
       <c r="I40" t="n">
-        <v>780</v>
+        <v>705</v>
       </c>
       <c r="J40" t="n">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="K40" t="n">
-        <v>63</v>
+        <v>52</v>
       </c>
       <c r="L40" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/ljf/reparacion-150j-10m-30_300tr-same_per_machined-780c_ljf.xlsx</t>
+          <t>Job To Machine/problemset/solution/ljf/reparacion-150j-10m-30_300tr-same_per_machined-705c_ljf.xlsx</t>
         </is>
       </c>
       <c r="M40" t="n">
-        <v>780</v>
+        <v>705</v>
       </c>
       <c r="N40" t="n">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="O40" t="n">
-        <v>63</v>
+        <v>52</v>
       </c>
     </row>
     <row r="41">
@@ -2740,49 +2740,49 @@
         </is>
       </c>
       <c r="C41" t="n">
-        <v>866</v>
+        <v>1660</v>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/mlf/reparacion-150j-10m-30_300tr-same_per_machined-866c_mlf.xlsx</t>
+          <t>Job To Machine/problemset/solution/mlf/reparacion-150j-10m-30_300tr-same_per_machined-1660.0c_mlf.xlsx</t>
         </is>
       </c>
       <c r="E41" t="n">
-        <v>865</v>
+        <v>1653</v>
       </c>
       <c r="F41" t="n">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="G41" t="n">
-        <v>68</v>
+        <v>130</v>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/sjf/reparacion-150j-10m-30_300tr-same_per_machined-866c_sjf.xlsx</t>
+          <t>Job To Machine/problemset/solution/sjf/reparacion-150j-10m-30_300tr-same_per_machined-1660.0c_sjf.xlsx</t>
         </is>
       </c>
       <c r="I41" t="n">
-        <v>865</v>
+        <v>1653</v>
       </c>
       <c r="J41" t="n">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="K41" t="n">
-        <v>68</v>
+        <v>130</v>
       </c>
       <c r="L41" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/ljf/reparacion-150j-10m-30_300tr-same_per_machined-866c_ljf.xlsx</t>
+          <t>Job To Machine/problemset/solution/ljf/reparacion-150j-10m-30_300tr-same_per_machined-1660.0c_ljf.xlsx</t>
         </is>
       </c>
       <c r="M41" t="n">
-        <v>865</v>
+        <v>1653</v>
       </c>
       <c r="N41" t="n">
-        <v>116</v>
+        <v>120</v>
       </c>
       <c r="O41" t="n">
-        <v>68</v>
+        <v>130</v>
       </c>
     </row>
     <row r="42">
@@ -2797,49 +2797,49 @@
         </is>
       </c>
       <c r="C42" t="n">
-        <v>2646</v>
+        <v>2486</v>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/mlf/reparacion-150j-10m-30_300tr-same_per_jobd-2646c_mlf.xlsx</t>
+          <t>Job To Machine/problemset/solution/mlf/reparacion-150j-10m-30_300tr-same_per_jobd-2486c_mlf.xlsx</t>
         </is>
       </c>
       <c r="E42" t="n">
-        <v>2643</v>
+        <v>2486</v>
       </c>
       <c r="F42" t="n">
-        <v>175</v>
+        <v>164</v>
       </c>
       <c r="G42" t="n">
         <v>149</v>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/sjf/reparacion-150j-10m-30_300tr-same_per_jobd-2646c_sjf.xlsx</t>
+          <t>Job To Machine/problemset/solution/sjf/reparacion-150j-10m-30_300tr-same_per_jobd-2486c_sjf.xlsx</t>
         </is>
       </c>
       <c r="I42" t="n">
-        <v>2643</v>
+        <v>2474</v>
       </c>
       <c r="J42" t="n">
-        <v>175</v>
+        <v>163</v>
       </c>
       <c r="K42" t="n">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="L42" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/ljf/reparacion-150j-10m-30_300tr-same_per_jobd-2646c_ljf.xlsx</t>
+          <t>Job To Machine/problemset/solution/ljf/reparacion-150j-10m-30_300tr-same_per_jobd-2486c_ljf.xlsx</t>
         </is>
       </c>
       <c r="M42" t="n">
-        <v>2643</v>
+        <v>2474</v>
       </c>
       <c r="N42" t="n">
-        <v>175</v>
+        <v>163</v>
       </c>
       <c r="O42" t="n">
-        <v>149</v>
+        <v>147</v>
       </c>
     </row>
     <row r="43">
@@ -2854,49 +2854,49 @@
         </is>
       </c>
       <c r="C43" t="n">
-        <v>2941</v>
+        <v>2487</v>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/mlf/reparacion-150j-10m-30_300tr-same_per_jobd-2941c_mlf.xlsx</t>
+          <t>Job To Machine/problemset/solution/mlf/reparacion-150j-10m-30_300tr-same_per_jobd-2487.0c_mlf.xlsx</t>
         </is>
       </c>
       <c r="E43" t="n">
-        <v>2941</v>
+        <v>2487</v>
       </c>
       <c r="F43" t="n">
-        <v>176</v>
+        <v>164</v>
       </c>
       <c r="G43" t="n">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/sjf/reparacion-150j-10m-30_300tr-same_per_jobd-2941c_sjf.xlsx</t>
+          <t>Job To Machine/problemset/solution/sjf/reparacion-150j-10m-30_300tr-same_per_jobd-2487.0c_sjf.xlsx</t>
         </is>
       </c>
       <c r="I43" t="n">
-        <v>2941</v>
+        <v>2474</v>
       </c>
       <c r="J43" t="n">
-        <v>176</v>
+        <v>163</v>
       </c>
       <c r="K43" t="n">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="L43" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/ljf/reparacion-150j-10m-30_300tr-same_per_jobd-2941c_ljf.xlsx</t>
+          <t>Job To Machine/problemset/solution/ljf/reparacion-150j-10m-30_300tr-same_per_jobd-2487.0c_ljf.xlsx</t>
         </is>
       </c>
       <c r="M43" t="n">
-        <v>2941</v>
+        <v>2474</v>
       </c>
       <c r="N43" t="n">
-        <v>176</v>
+        <v>163</v>
       </c>
       <c r="O43" t="n">
-        <v>150</v>
+        <v>147</v>
       </c>
     </row>
     <row r="44">
@@ -2911,49 +2911,49 @@
         </is>
       </c>
       <c r="C44" t="n">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/mlf/supermercado-150j-20m-5_20tr-uniformd-40c_mlf.xlsx</t>
+          <t>Job To Machine/problemset/solution/mlf/supermercado-150j-20m-5_20tr-uniformd-39c_mlf.xlsx</t>
         </is>
       </c>
       <c r="E44" t="n">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="F44" t="n">
         <v>5</v>
       </c>
       <c r="G44" t="n">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/sjf/supermercado-150j-20m-5_20tr-uniformd-40c_sjf.xlsx</t>
+          <t>Job To Machine/problemset/solution/sjf/supermercado-150j-20m-5_20tr-uniformd-39c_sjf.xlsx</t>
         </is>
       </c>
       <c r="I44" t="n">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="J44" t="n">
         <v>5</v>
       </c>
       <c r="K44" t="n">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="L44" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/ljf/supermercado-150j-20m-5_20tr-uniformd-40c_ljf.xlsx</t>
+          <t>Job To Machine/problemset/solution/ljf/supermercado-150j-20m-5_20tr-uniformd-39c_ljf.xlsx</t>
         </is>
       </c>
       <c r="M44" t="n">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="N44" t="n">
         <v>5</v>
       </c>
       <c r="O44" t="n">
-        <v>131</v>
+        <v>133</v>
       </c>
     </row>
     <row r="45">
@@ -2968,49 +2968,49 @@
         </is>
       </c>
       <c r="C45" t="n">
-        <v>42</v>
+        <v>60</v>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/mlf/supermercado-150j-20m-5_20tr-uniformd-42c_mlf.xlsx</t>
+          <t>Job To Machine/problemset/solution/mlf/supermercado-150j-20m-5_20tr-uniformd-60.0c_mlf.xlsx</t>
         </is>
       </c>
       <c r="E45" t="n">
-        <v>42</v>
+        <v>60</v>
       </c>
       <c r="F45" t="n">
         <v>5</v>
       </c>
       <c r="G45" t="n">
-        <v>140</v>
+        <v>150</v>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/sjf/supermercado-150j-20m-5_20tr-uniformd-42c_sjf.xlsx</t>
+          <t>Job To Machine/problemset/solution/sjf/supermercado-150j-20m-5_20tr-uniformd-60.0c_sjf.xlsx</t>
         </is>
       </c>
       <c r="I45" t="n">
-        <v>42</v>
+        <v>60</v>
       </c>
       <c r="J45" t="n">
         <v>5</v>
       </c>
       <c r="K45" t="n">
-        <v>140</v>
+        <v>150</v>
       </c>
       <c r="L45" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/ljf/supermercado-150j-20m-5_20tr-uniformd-42c_ljf.xlsx</t>
+          <t>Job To Machine/problemset/solution/ljf/supermercado-150j-20m-5_20tr-uniformd-60.0c_ljf.xlsx</t>
         </is>
       </c>
       <c r="M45" t="n">
-        <v>42</v>
+        <v>60</v>
       </c>
       <c r="N45" t="n">
         <v>5</v>
       </c>
       <c r="O45" t="n">
-        <v>140</v>
+        <v>150</v>
       </c>
     </row>
     <row r="46">
@@ -3082,11 +3082,11 @@
         </is>
       </c>
       <c r="C47" t="n">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/mlf/supermercado-150j-20m-5_20tr-constantd-39c_mlf.xlsx</t>
+          <t>Job To Machine/problemset/solution/mlf/supermercado-150j-20m-5_20tr-constantd-38.0c_mlf.xlsx</t>
         </is>
       </c>
       <c r="E47" t="n">
@@ -3100,7 +3100,7 @@
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/sjf/supermercado-150j-20m-5_20tr-constantd-39c_sjf.xlsx</t>
+          <t>Job To Machine/problemset/solution/sjf/supermercado-150j-20m-5_20tr-constantd-38.0c_sjf.xlsx</t>
         </is>
       </c>
       <c r="I47" t="n">
@@ -3114,7 +3114,7 @@
       </c>
       <c r="L47" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/ljf/supermercado-150j-20m-5_20tr-constantd-39c_ljf.xlsx</t>
+          <t>Job To Machine/problemset/solution/ljf/supermercado-150j-20m-5_20tr-constantd-38.0c_ljf.xlsx</t>
         </is>
       </c>
       <c r="M47" t="n">
@@ -3153,7 +3153,7 @@
         <v>6</v>
       </c>
       <c r="G48" t="n">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="H48" t="inlineStr">
         <is>
@@ -3164,10 +3164,10 @@
         <v>43</v>
       </c>
       <c r="J48" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="K48" t="n">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="L48" t="inlineStr">
         <is>
@@ -3181,7 +3181,7 @@
         <v>6</v>
       </c>
       <c r="O48" t="n">
-        <v>135</v>
+        <v>134</v>
       </c>
     </row>
     <row r="49">
@@ -3196,49 +3196,49 @@
         </is>
       </c>
       <c r="C49" t="n">
-        <v>45</v>
+        <v>69</v>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/mlf/supermercado-150j-20m-5_20tr-normald-45c_mlf.xlsx</t>
+          <t>Job To Machine/problemset/solution/mlf/supermercado-150j-20m-5_20tr-normald-69.0c_mlf.xlsx</t>
         </is>
       </c>
       <c r="E49" t="n">
-        <v>45</v>
+        <v>67</v>
       </c>
       <c r="F49" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="G49" t="n">
-        <v>142</v>
+        <v>150</v>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/sjf/supermercado-150j-20m-5_20tr-normald-45c_sjf.xlsx</t>
+          <t>Job To Machine/problemset/solution/sjf/supermercado-150j-20m-5_20tr-normald-69.0c_sjf.xlsx</t>
         </is>
       </c>
       <c r="I49" t="n">
-        <v>45</v>
+        <v>67</v>
       </c>
       <c r="J49" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="K49" t="n">
-        <v>142</v>
+        <v>150</v>
       </c>
       <c r="L49" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/ljf/supermercado-150j-20m-5_20tr-normald-45c_ljf.xlsx</t>
+          <t>Job To Machine/problemset/solution/ljf/supermercado-150j-20m-5_20tr-normald-69.0c_ljf.xlsx</t>
         </is>
       </c>
       <c r="M49" t="n">
-        <v>45</v>
+        <v>67</v>
       </c>
       <c r="N49" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="O49" t="n">
-        <v>142</v>
+        <v>150</v>
       </c>
     </row>
     <row r="50">
@@ -3267,7 +3267,7 @@
         <v>5</v>
       </c>
       <c r="G50" t="n">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="H50" t="inlineStr">
         <is>
@@ -3281,7 +3281,7 @@
         <v>5</v>
       </c>
       <c r="K50" t="n">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="L50" t="inlineStr">
         <is>
@@ -3310,49 +3310,49 @@
         </is>
       </c>
       <c r="C51" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/mlf/supermercado-150j-20m-5_20tr-exponentiald-39c_mlf.xlsx</t>
+          <t>Job To Machine/problemset/solution/mlf/supermercado-150j-20m-5_20tr-exponentiald-40.0c_mlf.xlsx</t>
         </is>
       </c>
       <c r="E51" t="n">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="F51" t="n">
         <v>5</v>
       </c>
       <c r="G51" t="n">
-        <v>139</v>
+        <v>150</v>
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/sjf/supermercado-150j-20m-5_20tr-exponentiald-39c_sjf.xlsx</t>
+          <t>Job To Machine/problemset/solution/sjf/supermercado-150j-20m-5_20tr-exponentiald-40.0c_sjf.xlsx</t>
         </is>
       </c>
       <c r="I51" t="n">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="J51" t="n">
         <v>5</v>
       </c>
       <c r="K51" t="n">
-        <v>139</v>
+        <v>150</v>
       </c>
       <c r="L51" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/ljf/supermercado-150j-20m-5_20tr-exponentiald-39c_ljf.xlsx</t>
+          <t>Job To Machine/problemset/solution/ljf/supermercado-150j-20m-5_20tr-exponentiald-40.0c_ljf.xlsx</t>
         </is>
       </c>
       <c r="M51" t="n">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="N51" t="n">
         <v>5</v>
       </c>
       <c r="O51" t="n">
-        <v>139</v>
+        <v>150</v>
       </c>
     </row>
     <row r="52">
@@ -3367,49 +3367,49 @@
         </is>
       </c>
       <c r="C52" t="n">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/mlf/supermercado-150j-20m-5_20tr-lognormald-46c_mlf.xlsx</t>
+          <t>Job To Machine/problemset/solution/mlf/supermercado-150j-20m-5_20tr-lognormald-43c_mlf.xlsx</t>
         </is>
       </c>
       <c r="E52" t="n">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="F52" t="n">
         <v>6</v>
       </c>
       <c r="G52" t="n">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/sjf/supermercado-150j-20m-5_20tr-lognormald-46c_sjf.xlsx</t>
+          <t>Job To Machine/problemset/solution/sjf/supermercado-150j-20m-5_20tr-lognormald-43c_sjf.xlsx</t>
         </is>
       </c>
       <c r="I52" t="n">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="J52" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="K52" t="n">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="L52" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/ljf/supermercado-150j-20m-5_20tr-lognormald-46c_ljf.xlsx</t>
+          <t>Job To Machine/problemset/solution/ljf/supermercado-150j-20m-5_20tr-lognormald-43c_ljf.xlsx</t>
         </is>
       </c>
       <c r="M52" t="n">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="N52" t="n">
         <v>6</v>
       </c>
       <c r="O52" t="n">
-        <v>138</v>
+        <v>134</v>
       </c>
     </row>
     <row r="53">
@@ -3424,49 +3424,49 @@
         </is>
       </c>
       <c r="C53" t="n">
-        <v>48</v>
+        <v>55</v>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/mlf/supermercado-150j-20m-5_20tr-lognormald-48c_mlf.xlsx</t>
+          <t>Job To Machine/problemset/solution/mlf/supermercado-150j-20m-5_20tr-lognormald-55.0c_mlf.xlsx</t>
         </is>
       </c>
       <c r="E53" t="n">
-        <v>48</v>
+        <v>55</v>
       </c>
       <c r="F53" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="G53" t="n">
-        <v>145</v>
+        <v>150</v>
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/sjf/supermercado-150j-20m-5_20tr-lognormald-48c_sjf.xlsx</t>
+          <t>Job To Machine/problemset/solution/sjf/supermercado-150j-20m-5_20tr-lognormald-55.0c_sjf.xlsx</t>
         </is>
       </c>
       <c r="I53" t="n">
-        <v>48</v>
+        <v>55</v>
       </c>
       <c r="J53" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="K53" t="n">
-        <v>145</v>
+        <v>150</v>
       </c>
       <c r="L53" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/ljf/supermercado-150j-20m-5_20tr-lognormald-48c_ljf.xlsx</t>
+          <t>Job To Machine/problemset/solution/ljf/supermercado-150j-20m-5_20tr-lognormald-55.0c_ljf.xlsx</t>
         </is>
       </c>
       <c r="M53" t="n">
-        <v>48</v>
+        <v>55</v>
       </c>
       <c r="N53" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="O53" t="n">
-        <v>145</v>
+        <v>150</v>
       </c>
     </row>
     <row r="54">
@@ -3492,10 +3492,10 @@
         <v>36</v>
       </c>
       <c r="F54" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="G54" t="n">
-        <v>60</v>
+        <v>69</v>
       </c>
       <c r="H54" t="inlineStr">
         <is>
@@ -3506,10 +3506,10 @@
         <v>36</v>
       </c>
       <c r="J54" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="K54" t="n">
-        <v>60</v>
+        <v>69</v>
       </c>
       <c r="L54" t="inlineStr">
         <is>
@@ -3520,10 +3520,10 @@
         <v>36</v>
       </c>
       <c r="N54" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="O54" t="n">
-        <v>60</v>
+        <v>69</v>
       </c>
     </row>
     <row r="55">
@@ -3538,49 +3538,49 @@
         </is>
       </c>
       <c r="C55" t="n">
-        <v>39</v>
+        <v>53</v>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/mlf/supermercado-150j-20m-5_20tr-same_per_machined-39c_mlf.xlsx</t>
+          <t>Job To Machine/problemset/solution/mlf/supermercado-150j-20m-5_20tr-same_per_machined-53.0c_mlf.xlsx</t>
         </is>
       </c>
       <c r="E55" t="n">
-        <v>39</v>
+        <v>52</v>
       </c>
       <c r="F55" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="G55" t="n">
-        <v>62</v>
+        <v>98</v>
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/sjf/supermercado-150j-20m-5_20tr-same_per_machined-39c_sjf.xlsx</t>
+          <t>Job To Machine/problemset/solution/sjf/supermercado-150j-20m-5_20tr-same_per_machined-53.0c_sjf.xlsx</t>
         </is>
       </c>
       <c r="I55" t="n">
-        <v>39</v>
+        <v>52</v>
       </c>
       <c r="J55" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="K55" t="n">
-        <v>62</v>
+        <v>98</v>
       </c>
       <c r="L55" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/ljf/supermercado-150j-20m-5_20tr-same_per_machined-39c_ljf.xlsx</t>
+          <t>Job To Machine/problemset/solution/ljf/supermercado-150j-20m-5_20tr-same_per_machined-53.0c_ljf.xlsx</t>
         </is>
       </c>
       <c r="M55" t="n">
-        <v>39</v>
+        <v>52</v>
       </c>
       <c r="N55" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="O55" t="n">
-        <v>62</v>
+        <v>98</v>
       </c>
     </row>
     <row r="56">
@@ -3595,49 +3595,49 @@
         </is>
       </c>
       <c r="C56" t="n">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/mlf/supermercado-150j-20m-5_20tr-same_per_jobd-84c_mlf.xlsx</t>
+          <t>Job To Machine/problemset/solution/mlf/supermercado-150j-20m-5_20tr-same_per_jobd-88c_mlf.xlsx</t>
         </is>
       </c>
       <c r="E56" t="n">
-        <v>84</v>
+        <v>88</v>
       </c>
       <c r="F56" t="n">
         <v>11</v>
       </c>
       <c r="G56" t="n">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/sjf/supermercado-150j-20m-5_20tr-same_per_jobd-84c_sjf.xlsx</t>
+          <t>Job To Machine/problemset/solution/sjf/supermercado-150j-20m-5_20tr-same_per_jobd-88c_sjf.xlsx</t>
         </is>
       </c>
       <c r="I56" t="n">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="J56" t="n">
         <v>11</v>
       </c>
       <c r="K56" t="n">
-        <v>148</v>
+        <v>141</v>
       </c>
       <c r="L56" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/ljf/supermercado-150j-20m-5_20tr-same_per_jobd-84c_ljf.xlsx</t>
+          <t>Job To Machine/problemset/solution/ljf/supermercado-150j-20m-5_20tr-same_per_jobd-88c_ljf.xlsx</t>
         </is>
       </c>
       <c r="M56" t="n">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="N56" t="n">
         <v>11</v>
       </c>
       <c r="O56" t="n">
-        <v>148</v>
+        <v>141</v>
       </c>
     </row>
     <row r="57">
@@ -3652,49 +3652,49 @@
         </is>
       </c>
       <c r="C57" t="n">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/mlf/supermercado-150j-20m-5_20tr-same_per_jobd-88c_mlf.xlsx</t>
+          <t>Job To Machine/problemset/solution/mlf/supermercado-150j-20m-5_20tr-same_per_jobd-89.0c_mlf.xlsx</t>
         </is>
       </c>
       <c r="E57" t="n">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="F57" t="n">
         <v>11</v>
       </c>
       <c r="G57" t="n">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/sjf/supermercado-150j-20m-5_20tr-same_per_jobd-88c_sjf.xlsx</t>
+          <t>Job To Machine/problemset/solution/sjf/supermercado-150j-20m-5_20tr-same_per_jobd-89.0c_sjf.xlsx</t>
         </is>
       </c>
       <c r="I57" t="n">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="J57" t="n">
         <v>11</v>
       </c>
       <c r="K57" t="n">
-        <v>150</v>
+        <v>142</v>
       </c>
       <c r="L57" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/ljf/supermercado-150j-20m-5_20tr-same_per_jobd-88c_ljf.xlsx</t>
+          <t>Job To Machine/problemset/solution/ljf/supermercado-150j-20m-5_20tr-same_per_jobd-89.0c_ljf.xlsx</t>
         </is>
       </c>
       <c r="M57" t="n">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="N57" t="n">
         <v>11</v>
       </c>
       <c r="O57" t="n">
-        <v>150</v>
+        <v>142</v>
       </c>
     </row>
     <row r="58">
@@ -3723,7 +3723,7 @@
         <v>2</v>
       </c>
       <c r="G58" t="n">
-        <v>901</v>
+        <v>903</v>
       </c>
       <c r="H58" t="inlineStr">
         <is>
@@ -3737,7 +3737,7 @@
         <v>2</v>
       </c>
       <c r="K58" t="n">
-        <v>901</v>
+        <v>912</v>
       </c>
       <c r="L58" t="inlineStr">
         <is>
@@ -3751,7 +3751,7 @@
         <v>2</v>
       </c>
       <c r="O58" t="n">
-        <v>901</v>
+        <v>900</v>
       </c>
     </row>
     <row r="59">
@@ -3766,49 +3766,49 @@
         </is>
       </c>
       <c r="C59" t="n">
-        <v>20</v>
+        <v>73</v>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/mlf/call_center-1000j-100m-2_30tr-uniformd-20c_mlf.xlsx</t>
+          <t>Job To Machine/problemset/solution/mlf/call_center-1000j-100m-2_30tr-uniformd-73.0c_mlf.xlsx</t>
         </is>
       </c>
       <c r="E59" t="n">
-        <v>20</v>
+        <v>70</v>
       </c>
       <c r="F59" t="n">
         <v>2</v>
       </c>
       <c r="G59" t="n">
-        <v>901</v>
+        <v>1000</v>
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/sjf/call_center-1000j-100m-2_30tr-uniformd-20c_sjf.xlsx</t>
+          <t>Job To Machine/problemset/solution/sjf/call_center-1000j-100m-2_30tr-uniformd-73.0c_sjf.xlsx</t>
         </is>
       </c>
       <c r="I59" t="n">
-        <v>20</v>
+        <v>70</v>
       </c>
       <c r="J59" t="n">
         <v>2</v>
       </c>
       <c r="K59" t="n">
-        <v>901</v>
+        <v>1000</v>
       </c>
       <c r="L59" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/ljf/call_center-1000j-100m-2_30tr-uniformd-20c_ljf.xlsx</t>
+          <t>Job To Machine/problemset/solution/ljf/call_center-1000j-100m-2_30tr-uniformd-73.0c_ljf.xlsx</t>
         </is>
       </c>
       <c r="M59" t="n">
-        <v>20</v>
+        <v>70</v>
       </c>
       <c r="N59" t="n">
         <v>2</v>
       </c>
       <c r="O59" t="n">
-        <v>901</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="60">
@@ -3884,7 +3884,7 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/mlf/call_center-1000j-100m-2_30tr-constantd-20c_mlf.xlsx</t>
+          <t>Job To Machine/problemset/solution/mlf/call_center-1000j-100m-2_30tr-constantd-20.0c_mlf.xlsx</t>
         </is>
       </c>
       <c r="E61" t="n">
@@ -3898,7 +3898,7 @@
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/sjf/call_center-1000j-100m-2_30tr-constantd-20c_sjf.xlsx</t>
+          <t>Job To Machine/problemset/solution/sjf/call_center-1000j-100m-2_30tr-constantd-20.0c_sjf.xlsx</t>
         </is>
       </c>
       <c r="I61" t="n">
@@ -3912,7 +3912,7 @@
       </c>
       <c r="L61" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/ljf/call_center-1000j-100m-2_30tr-constantd-20c_ljf.xlsx</t>
+          <t>Job To Machine/problemset/solution/ljf/call_center-1000j-100m-2_30tr-constantd-20.0c_ljf.xlsx</t>
         </is>
       </c>
       <c r="M61" t="n">
@@ -3951,7 +3951,7 @@
         <v>2</v>
       </c>
       <c r="G62" t="n">
-        <v>860</v>
+        <v>867</v>
       </c>
       <c r="H62" t="inlineStr">
         <is>
@@ -3965,7 +3965,7 @@
         <v>2</v>
       </c>
       <c r="K62" t="n">
-        <v>860</v>
+        <v>883</v>
       </c>
       <c r="L62" t="inlineStr">
         <is>
@@ -3979,7 +3979,7 @@
         <v>2</v>
       </c>
       <c r="O62" t="n">
-        <v>860</v>
+        <v>873</v>
       </c>
     </row>
     <row r="63">
@@ -3994,49 +3994,49 @@
         </is>
       </c>
       <c r="C63" t="n">
-        <v>20</v>
+        <v>97</v>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/mlf/call_center-1000j-100m-2_30tr-normald-20c_mlf.xlsx</t>
+          <t>Job To Machine/problemset/solution/mlf/call_center-1000j-100m-2_30tr-normald-97.0c_mlf.xlsx</t>
         </is>
       </c>
       <c r="E63" t="n">
-        <v>20</v>
+        <v>76</v>
       </c>
       <c r="F63" t="n">
         <v>2</v>
       </c>
       <c r="G63" t="n">
-        <v>860</v>
+        <v>1000</v>
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/sjf/call_center-1000j-100m-2_30tr-normald-20c_sjf.xlsx</t>
+          <t>Job To Machine/problemset/solution/sjf/call_center-1000j-100m-2_30tr-normald-97.0c_sjf.xlsx</t>
         </is>
       </c>
       <c r="I63" t="n">
-        <v>20</v>
+        <v>76</v>
       </c>
       <c r="J63" t="n">
         <v>2</v>
       </c>
       <c r="K63" t="n">
-        <v>860</v>
+        <v>1000</v>
       </c>
       <c r="L63" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/ljf/call_center-1000j-100m-2_30tr-normald-20c_ljf.xlsx</t>
+          <t>Job To Machine/problemset/solution/ljf/call_center-1000j-100m-2_30tr-normald-97.0c_ljf.xlsx</t>
         </is>
       </c>
       <c r="M63" t="n">
-        <v>20</v>
+        <v>76</v>
       </c>
       <c r="N63" t="n">
         <v>2</v>
       </c>
       <c r="O63" t="n">
-        <v>860</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="64">
@@ -4065,7 +4065,7 @@
         <v>2</v>
       </c>
       <c r="G64" t="n">
-        <v>989</v>
+        <v>993</v>
       </c>
       <c r="H64" t="inlineStr">
         <is>
@@ -4079,7 +4079,7 @@
         <v>2</v>
       </c>
       <c r="K64" t="n">
-        <v>989</v>
+        <v>993</v>
       </c>
       <c r="L64" t="inlineStr">
         <is>
@@ -4093,7 +4093,7 @@
         <v>2</v>
       </c>
       <c r="O64" t="n">
-        <v>989</v>
+        <v>992</v>
       </c>
     </row>
     <row r="65">
@@ -4108,49 +4108,49 @@
         </is>
       </c>
       <c r="C65" t="n">
-        <v>20</v>
+        <v>29</v>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/mlf/call_center-1000j-100m-2_30tr-exponentiald-20c_mlf.xlsx</t>
+          <t>Job To Machine/problemset/solution/mlf/call_center-1000j-100m-2_30tr-exponentiald-29.0c_mlf.xlsx</t>
         </is>
       </c>
       <c r="E65" t="n">
-        <v>20</v>
+        <v>28</v>
       </c>
       <c r="F65" t="n">
         <v>2</v>
       </c>
       <c r="G65" t="n">
-        <v>989</v>
+        <v>1000</v>
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/sjf/call_center-1000j-100m-2_30tr-exponentiald-20c_sjf.xlsx</t>
+          <t>Job To Machine/problemset/solution/sjf/call_center-1000j-100m-2_30tr-exponentiald-29.0c_sjf.xlsx</t>
         </is>
       </c>
       <c r="I65" t="n">
-        <v>20</v>
+        <v>28</v>
       </c>
       <c r="J65" t="n">
         <v>2</v>
       </c>
       <c r="K65" t="n">
-        <v>989</v>
+        <v>1000</v>
       </c>
       <c r="L65" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/ljf/call_center-1000j-100m-2_30tr-exponentiald-20c_ljf.xlsx</t>
+          <t>Job To Machine/problemset/solution/ljf/call_center-1000j-100m-2_30tr-exponentiald-29.0c_ljf.xlsx</t>
         </is>
       </c>
       <c r="M65" t="n">
-        <v>20</v>
+        <v>28</v>
       </c>
       <c r="N65" t="n">
         <v>2</v>
       </c>
       <c r="O65" t="n">
-        <v>989</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="66">
@@ -4165,49 +4165,49 @@
         </is>
       </c>
       <c r="C66" t="n">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/mlf/call_center-1000j-100m-2_30tr-lognormald-37c_mlf.xlsx</t>
+          <t>Job To Machine/problemset/solution/mlf/call_center-1000j-100m-2_30tr-lognormald-33c_mlf.xlsx</t>
         </is>
       </c>
       <c r="E66" t="n">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="F66" t="n">
         <v>3</v>
       </c>
       <c r="G66" t="n">
-        <v>929</v>
+        <v>899</v>
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/sjf/call_center-1000j-100m-2_30tr-lognormald-37c_sjf.xlsx</t>
+          <t>Job To Machine/problemset/solution/sjf/call_center-1000j-100m-2_30tr-lognormald-33c_sjf.xlsx</t>
         </is>
       </c>
       <c r="I66" t="n">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="J66" t="n">
         <v>3</v>
       </c>
       <c r="K66" t="n">
-        <v>929</v>
+        <v>926</v>
       </c>
       <c r="L66" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/ljf/call_center-1000j-100m-2_30tr-lognormald-37c_ljf.xlsx</t>
+          <t>Job To Machine/problemset/solution/ljf/call_center-1000j-100m-2_30tr-lognormald-33c_ljf.xlsx</t>
         </is>
       </c>
       <c r="M66" t="n">
-        <v>37</v>
+        <v>33</v>
       </c>
       <c r="N66" t="n">
         <v>3</v>
       </c>
       <c r="O66" t="n">
-        <v>929</v>
+        <v>909</v>
       </c>
     </row>
     <row r="67">
@@ -4222,49 +4222,49 @@
         </is>
       </c>
       <c r="C67" t="n">
-        <v>37</v>
+        <v>62</v>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/mlf/call_center-1000j-100m-2_30tr-lognormald-37c_mlf.xlsx</t>
+          <t>Job To Machine/problemset/solution/mlf/call_center-1000j-100m-2_30tr-lognormald-62.0c_mlf.xlsx</t>
         </is>
       </c>
       <c r="E67" t="n">
-        <v>37</v>
+        <v>62</v>
       </c>
       <c r="F67" t="n">
         <v>3</v>
       </c>
       <c r="G67" t="n">
-        <v>929</v>
+        <v>1000</v>
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/sjf/call_center-1000j-100m-2_30tr-lognormald-37c_sjf.xlsx</t>
+          <t>Job To Machine/problemset/solution/sjf/call_center-1000j-100m-2_30tr-lognormald-62.0c_sjf.xlsx</t>
         </is>
       </c>
       <c r="I67" t="n">
-        <v>37</v>
+        <v>62</v>
       </c>
       <c r="J67" t="n">
         <v>3</v>
       </c>
       <c r="K67" t="n">
-        <v>929</v>
+        <v>1000</v>
       </c>
       <c r="L67" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/ljf/call_center-1000j-100m-2_30tr-lognormald-37c_ljf.xlsx</t>
+          <t>Job To Machine/problemset/solution/ljf/call_center-1000j-100m-2_30tr-lognormald-62.0c_ljf.xlsx</t>
         </is>
       </c>
       <c r="M67" t="n">
-        <v>37</v>
+        <v>62</v>
       </c>
       <c r="N67" t="n">
         <v>3</v>
       </c>
       <c r="O67" t="n">
-        <v>929</v>
+        <v>1000</v>
       </c>
     </row>
     <row r="68">
@@ -4290,10 +4290,10 @@
         <v>20</v>
       </c>
       <c r="F68" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G68" t="n">
-        <v>192</v>
+        <v>141</v>
       </c>
       <c r="H68" t="inlineStr">
         <is>
@@ -4304,10 +4304,10 @@
         <v>20</v>
       </c>
       <c r="J68" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="K68" t="n">
-        <v>192</v>
+        <v>141</v>
       </c>
       <c r="L68" t="inlineStr">
         <is>
@@ -4318,10 +4318,10 @@
         <v>20</v>
       </c>
       <c r="N68" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="O68" t="n">
-        <v>192</v>
+        <v>141</v>
       </c>
     </row>
     <row r="69">
@@ -4336,49 +4336,49 @@
         </is>
       </c>
       <c r="C69" t="n">
-        <v>20</v>
+        <v>78</v>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/mlf/call_center-1000j-100m-2_30tr-same_per_machined-20c_mlf.xlsx</t>
+          <t>Job To Machine/problemset/solution/mlf/call_center-1000j-100m-2_30tr-same_per_machined-78.0c_mlf.xlsx</t>
         </is>
       </c>
       <c r="E69" t="n">
-        <v>20</v>
+        <v>78</v>
       </c>
       <c r="F69" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="G69" t="n">
-        <v>192</v>
+        <v>694</v>
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/sjf/call_center-1000j-100m-2_30tr-same_per_machined-20c_sjf.xlsx</t>
+          <t>Job To Machine/problemset/solution/sjf/call_center-1000j-100m-2_30tr-same_per_machined-78.0c_sjf.xlsx</t>
         </is>
       </c>
       <c r="I69" t="n">
-        <v>20</v>
+        <v>78</v>
       </c>
       <c r="J69" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="K69" t="n">
-        <v>192</v>
+        <v>694</v>
       </c>
       <c r="L69" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/ljf/call_center-1000j-100m-2_30tr-same_per_machined-20c_ljf.xlsx</t>
+          <t>Job To Machine/problemset/solution/ljf/call_center-1000j-100m-2_30tr-same_per_machined-78.0c_ljf.xlsx</t>
         </is>
       </c>
       <c r="M69" t="n">
-        <v>20</v>
+        <v>78</v>
       </c>
       <c r="N69" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="O69" t="n">
-        <v>192</v>
+        <v>694</v>
       </c>
     </row>
     <row r="70">
@@ -4393,49 +4393,49 @@
         </is>
       </c>
       <c r="C70" t="n">
-        <v>155</v>
+        <v>159</v>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/mlf/call_center-1000j-100m-2_30tr-same_per_jobd-155c_mlf.xlsx</t>
+          <t>Job To Machine/problemset/solution/mlf/call_center-1000j-100m-2_30tr-same_per_jobd-159c_mlf.xlsx</t>
         </is>
       </c>
       <c r="E70" t="n">
-        <v>155</v>
+        <v>159</v>
       </c>
       <c r="F70" t="n">
         <v>15</v>
       </c>
       <c r="G70" t="n">
-        <v>993</v>
+        <v>994</v>
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/sjf/call_center-1000j-100m-2_30tr-same_per_jobd-155c_sjf.xlsx</t>
+          <t>Job To Machine/problemset/solution/sjf/call_center-1000j-100m-2_30tr-same_per_jobd-159c_sjf.xlsx</t>
         </is>
       </c>
       <c r="I70" t="n">
-        <v>155</v>
+        <v>159</v>
       </c>
       <c r="J70" t="n">
         <v>15</v>
       </c>
       <c r="K70" t="n">
-        <v>993</v>
+        <v>958</v>
       </c>
       <c r="L70" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/ljf/call_center-1000j-100m-2_30tr-same_per_jobd-155c_ljf.xlsx</t>
+          <t>Job To Machine/problemset/solution/ljf/call_center-1000j-100m-2_30tr-same_per_jobd-159c_ljf.xlsx</t>
         </is>
       </c>
       <c r="M70" t="n">
-        <v>155</v>
+        <v>159</v>
       </c>
       <c r="N70" t="n">
         <v>15</v>
       </c>
       <c r="O70" t="n">
-        <v>993</v>
+        <v>958</v>
       </c>
     </row>
     <row r="71">
@@ -4450,49 +4450,49 @@
         </is>
       </c>
       <c r="C71" t="n">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/mlf/call_center-1000j-100m-2_30tr-same_per_jobd-157c_mlf.xlsx</t>
+          <t>Job To Machine/problemset/solution/mlf/call_center-1000j-100m-2_30tr-same_per_jobd-160.0c_mlf.xlsx</t>
         </is>
       </c>
       <c r="E71" t="n">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="F71" t="n">
         <v>15</v>
       </c>
       <c r="G71" t="n">
-        <v>1000</v>
+        <v>999</v>
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/sjf/call_center-1000j-100m-2_30tr-same_per_jobd-157c_sjf.xlsx</t>
+          <t>Job To Machine/problemset/solution/sjf/call_center-1000j-100m-2_30tr-same_per_jobd-160.0c_sjf.xlsx</t>
         </is>
       </c>
       <c r="I71" t="n">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="J71" t="n">
         <v>15</v>
       </c>
       <c r="K71" t="n">
-        <v>1000</v>
+        <v>964</v>
       </c>
       <c r="L71" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/ljf/call_center-1000j-100m-2_30tr-same_per_jobd-157c_ljf.xlsx</t>
+          <t>Job To Machine/problemset/solution/ljf/call_center-1000j-100m-2_30tr-same_per_jobd-160.0c_ljf.xlsx</t>
         </is>
       </c>
       <c r="M71" t="n">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="N71" t="n">
         <v>15</v>
       </c>
       <c r="O71" t="n">
-        <v>1000</v>
+        <v>964</v>
       </c>
     </row>
     <row r="72">
@@ -4507,49 +4507,49 @@
         </is>
       </c>
       <c r="C72" t="n">
-        <v>4014</v>
+        <v>4065</v>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/mlf/metalurgia-10000j-50m-1_1000tr-uniformd-4014c_mlf.xlsx</t>
+          <t>Job To Machine/problemset/solution/mlf/metalurgia-10000j-50m-1_1000tr-uniformd-4065c_mlf.xlsx</t>
         </is>
       </c>
       <c r="E72" t="n">
-        <v>4014</v>
+        <v>4065</v>
       </c>
       <c r="F72" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="G72" t="n">
-        <v>9586</v>
+        <v>9639</v>
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/sjf/metalurgia-10000j-50m-1_1000tr-uniformd-4014c_sjf.xlsx</t>
+          <t>Job To Machine/problemset/solution/sjf/metalurgia-10000j-50m-1_1000tr-uniformd-4065c_sjf.xlsx</t>
         </is>
       </c>
       <c r="I72" t="n">
-        <v>4014</v>
+        <v>4064</v>
       </c>
       <c r="J72" t="n">
         <v>20</v>
       </c>
       <c r="K72" t="n">
-        <v>9586</v>
+        <v>9955</v>
       </c>
       <c r="L72" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/ljf/metalurgia-10000j-50m-1_1000tr-uniformd-4014c_ljf.xlsx</t>
+          <t>Job To Machine/problemset/solution/ljf/metalurgia-10000j-50m-1_1000tr-uniformd-4065c_ljf.xlsx</t>
         </is>
       </c>
       <c r="M72" t="n">
-        <v>4014</v>
+        <v>4065</v>
       </c>
       <c r="N72" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="O72" t="n">
-        <v>9586</v>
+        <v>9645</v>
       </c>
     </row>
     <row r="73">
@@ -4564,49 +4564,49 @@
         </is>
       </c>
       <c r="C73" t="n">
-        <v>4096</v>
+        <v>42332</v>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/mlf/metalurgia-10000j-50m-1_1000tr-uniformd-4096c_mlf.xlsx</t>
+          <t>Job To Machine/problemset/solution/mlf/metalurgia-10000j-50m-1_1000tr-uniformd-42332.0c_mlf.xlsx</t>
         </is>
       </c>
       <c r="E73" t="n">
-        <v>4096</v>
+        <v>4837</v>
       </c>
       <c r="F73" t="n">
         <v>20</v>
       </c>
       <c r="G73" t="n">
-        <v>9811</v>
+        <v>10000</v>
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/sjf/metalurgia-10000j-50m-1_1000tr-uniformd-4096c_sjf.xlsx</t>
+          <t>Job To Machine/problemset/solution/sjf/metalurgia-10000j-50m-1_1000tr-uniformd-42332.0c_sjf.xlsx</t>
         </is>
       </c>
       <c r="I73" t="n">
-        <v>4096</v>
+        <v>4837</v>
       </c>
       <c r="J73" t="n">
         <v>20</v>
       </c>
       <c r="K73" t="n">
-        <v>9811</v>
+        <v>10000</v>
       </c>
       <c r="L73" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/ljf/metalurgia-10000j-50m-1_1000tr-uniformd-4096c_ljf.xlsx</t>
+          <t>Job To Machine/problemset/solution/ljf/metalurgia-10000j-50m-1_1000tr-uniformd-42332.0c_ljf.xlsx</t>
         </is>
       </c>
       <c r="M73" t="n">
-        <v>4096</v>
+        <v>4837</v>
       </c>
       <c r="N73" t="n">
         <v>20</v>
       </c>
       <c r="O73" t="n">
-        <v>9811</v>
+        <v>10000</v>
       </c>
     </row>
     <row r="74">
@@ -4678,15 +4678,15 @@
         </is>
       </c>
       <c r="C75" t="n">
-        <v>204</v>
+        <v>200</v>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/mlf/metalurgia-10000j-50m-1_1000tr-constantd-204c_mlf.xlsx</t>
+          <t>Job To Machine/problemset/solution/mlf/metalurgia-10000j-50m-1_1000tr-constantd-200.0c_mlf.xlsx</t>
         </is>
       </c>
       <c r="E75" t="n">
-        <v>204</v>
+        <v>200</v>
       </c>
       <c r="F75" t="n">
         <v>1</v>
@@ -4696,11 +4696,11 @@
       </c>
       <c r="H75" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/sjf/metalurgia-10000j-50m-1_1000tr-constantd-204c_sjf.xlsx</t>
+          <t>Job To Machine/problemset/solution/sjf/metalurgia-10000j-50m-1_1000tr-constantd-200.0c_sjf.xlsx</t>
         </is>
       </c>
       <c r="I75" t="n">
-        <v>204</v>
+        <v>200</v>
       </c>
       <c r="J75" t="n">
         <v>1</v>
@@ -4710,11 +4710,11 @@
       </c>
       <c r="L75" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/ljf/metalurgia-10000j-50m-1_1000tr-constantd-204c_ljf.xlsx</t>
+          <t>Job To Machine/problemset/solution/ljf/metalurgia-10000j-50m-1_1000tr-constantd-200.0c_ljf.xlsx</t>
         </is>
       </c>
       <c r="M75" t="n">
-        <v>204</v>
+        <v>200</v>
       </c>
       <c r="N75" t="n">
         <v>1</v>
@@ -4735,49 +4735,49 @@
         </is>
       </c>
       <c r="C76" t="n">
-        <v>4080</v>
+        <v>4006</v>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/mlf/metalurgia-10000j-50m-1_1000tr-normald-4080c_mlf.xlsx</t>
+          <t>Job To Machine/problemset/solution/mlf/metalurgia-10000j-50m-1_1000tr-normald-4006c_mlf.xlsx</t>
         </is>
       </c>
       <c r="E76" t="n">
-        <v>4080</v>
+        <v>4006</v>
       </c>
       <c r="F76" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="G76" t="n">
-        <v>9653</v>
+        <v>9716</v>
       </c>
       <c r="H76" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/sjf/metalurgia-10000j-50m-1_1000tr-normald-4080c_sjf.xlsx</t>
+          <t>Job To Machine/problemset/solution/sjf/metalurgia-10000j-50m-1_1000tr-normald-4006c_sjf.xlsx</t>
         </is>
       </c>
       <c r="I76" t="n">
-        <v>4080</v>
+        <v>4005</v>
       </c>
       <c r="J76" t="n">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="K76" t="n">
-        <v>9653</v>
+        <v>9962</v>
       </c>
       <c r="L76" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/ljf/metalurgia-10000j-50m-1_1000tr-normald-4080c_ljf.xlsx</t>
+          <t>Job To Machine/problemset/solution/ljf/metalurgia-10000j-50m-1_1000tr-normald-4006c_ljf.xlsx</t>
         </is>
       </c>
       <c r="M76" t="n">
-        <v>4080</v>
+        <v>4006</v>
       </c>
       <c r="N76" t="n">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="O76" t="n">
-        <v>9653</v>
+        <v>9954</v>
       </c>
     </row>
     <row r="77">
@@ -4792,49 +4792,49 @@
         </is>
       </c>
       <c r="C77" t="n">
-        <v>4163</v>
+        <v>59169</v>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/mlf/metalurgia-10000j-50m-1_1000tr-normald-4163c_mlf.xlsx</t>
+          <t>Job To Machine/problemset/solution/mlf/metalurgia-10000j-50m-1_1000tr-normald-59169.0c_mlf.xlsx</t>
         </is>
       </c>
       <c r="E77" t="n">
-        <v>4163</v>
+        <v>5524</v>
       </c>
       <c r="F77" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="G77" t="n">
-        <v>9796</v>
+        <v>10000</v>
       </c>
       <c r="H77" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/sjf/metalurgia-10000j-50m-1_1000tr-normald-4163c_sjf.xlsx</t>
+          <t>Job To Machine/problemset/solution/sjf/metalurgia-10000j-50m-1_1000tr-normald-59169.0c_sjf.xlsx</t>
         </is>
       </c>
       <c r="I77" t="n">
-        <v>4163</v>
+        <v>5524</v>
       </c>
       <c r="J77" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="K77" t="n">
-        <v>9796</v>
+        <v>10000</v>
       </c>
       <c r="L77" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/ljf/metalurgia-10000j-50m-1_1000tr-normald-4163c_ljf.xlsx</t>
+          <t>Job To Machine/problemset/solution/ljf/metalurgia-10000j-50m-1_1000tr-normald-59169.0c_ljf.xlsx</t>
         </is>
       </c>
       <c r="M77" t="n">
-        <v>4163</v>
+        <v>5524</v>
       </c>
       <c r="N77" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="O77" t="n">
-        <v>9796</v>
+        <v>10000</v>
       </c>
     </row>
     <row r="78">
@@ -4849,49 +4849,49 @@
         </is>
       </c>
       <c r="C78" t="n">
-        <v>909</v>
+        <v>908</v>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/mlf/metalurgia-10000j-50m-1_1000tr-exponentiald-909c_mlf.xlsx</t>
+          <t>Job To Machine/problemset/solution/mlf/metalurgia-10000j-50m-1_1000tr-exponentiald-908c_mlf.xlsx</t>
         </is>
       </c>
       <c r="E78" t="n">
-        <v>909</v>
+        <v>908</v>
       </c>
       <c r="F78" t="n">
         <v>4</v>
       </c>
       <c r="G78" t="n">
-        <v>9607</v>
+        <v>9547</v>
       </c>
       <c r="H78" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/sjf/metalurgia-10000j-50m-1_1000tr-exponentiald-909c_sjf.xlsx</t>
+          <t>Job To Machine/problemset/solution/sjf/metalurgia-10000j-50m-1_1000tr-exponentiald-908c_sjf.xlsx</t>
         </is>
       </c>
       <c r="I78" t="n">
-        <v>909</v>
+        <v>908</v>
       </c>
       <c r="J78" t="n">
         <v>4</v>
       </c>
       <c r="K78" t="n">
-        <v>9607</v>
+        <v>9939</v>
       </c>
       <c r="L78" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/ljf/metalurgia-10000j-50m-1_1000tr-exponentiald-909c_ljf.xlsx</t>
+          <t>Job To Machine/problemset/solution/ljf/metalurgia-10000j-50m-1_1000tr-exponentiald-908c_ljf.xlsx</t>
         </is>
       </c>
       <c r="M78" t="n">
-        <v>909</v>
+        <v>908</v>
       </c>
       <c r="N78" t="n">
         <v>4</v>
       </c>
       <c r="O78" t="n">
-        <v>9607</v>
+        <v>9692</v>
       </c>
     </row>
     <row r="79">
@@ -4906,49 +4906,49 @@
         </is>
       </c>
       <c r="C79" t="n">
-        <v>927</v>
+        <v>9731</v>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/mlf/metalurgia-10000j-50m-1_1000tr-exponentiald-927c_mlf.xlsx</t>
+          <t>Job To Machine/problemset/solution/mlf/metalurgia-10000j-50m-1_1000tr-exponentiald-9731.0c_mlf.xlsx</t>
         </is>
       </c>
       <c r="E79" t="n">
-        <v>927</v>
+        <v>1123</v>
       </c>
       <c r="F79" t="n">
         <v>4</v>
       </c>
       <c r="G79" t="n">
-        <v>9801</v>
+        <v>10000</v>
       </c>
       <c r="H79" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/sjf/metalurgia-10000j-50m-1_1000tr-exponentiald-927c_sjf.xlsx</t>
+          <t>Job To Machine/problemset/solution/sjf/metalurgia-10000j-50m-1_1000tr-exponentiald-9731.0c_sjf.xlsx</t>
         </is>
       </c>
       <c r="I79" t="n">
-        <v>927</v>
+        <v>1123</v>
       </c>
       <c r="J79" t="n">
         <v>4</v>
       </c>
       <c r="K79" t="n">
-        <v>9801</v>
+        <v>10000</v>
       </c>
       <c r="L79" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/ljf/metalurgia-10000j-50m-1_1000tr-exponentiald-927c_ljf.xlsx</t>
+          <t>Job To Machine/problemset/solution/ljf/metalurgia-10000j-50m-1_1000tr-exponentiald-9731.0c_ljf.xlsx</t>
         </is>
       </c>
       <c r="M79" t="n">
-        <v>927</v>
+        <v>1123</v>
       </c>
       <c r="N79" t="n">
         <v>4</v>
       </c>
       <c r="O79" t="n">
-        <v>9801</v>
+        <v>10000</v>
       </c>
     </row>
     <row r="80">
@@ -4963,49 +4963,49 @@
         </is>
       </c>
       <c r="C80" t="n">
-        <v>19862</v>
+        <v>19259</v>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/mlf/metalurgia-10000j-50m-1_1000tr-lognormald-19862c_mlf.xlsx</t>
+          <t>Job To Machine/problemset/solution/mlf/metalurgia-10000j-50m-1_1000tr-lognormald-19259c_mlf.xlsx</t>
         </is>
       </c>
       <c r="E80" t="n">
-        <v>19862</v>
+        <v>19259</v>
       </c>
       <c r="F80" t="n">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="G80" t="n">
-        <v>9866</v>
+        <v>9850</v>
       </c>
       <c r="H80" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/sjf/metalurgia-10000j-50m-1_1000tr-lognormald-19862c_sjf.xlsx</t>
+          <t>Job To Machine/problemset/solution/sjf/metalurgia-10000j-50m-1_1000tr-lognormald-19259c_sjf.xlsx</t>
         </is>
       </c>
       <c r="I80" t="n">
-        <v>19862</v>
+        <v>19259</v>
       </c>
       <c r="J80" t="n">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="K80" t="n">
-        <v>9866</v>
+        <v>9944</v>
       </c>
       <c r="L80" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/ljf/metalurgia-10000j-50m-1_1000tr-lognormald-19862c_ljf.xlsx</t>
+          <t>Job To Machine/problemset/solution/ljf/metalurgia-10000j-50m-1_1000tr-lognormald-19259c_ljf.xlsx</t>
         </is>
       </c>
       <c r="M80" t="n">
-        <v>19862</v>
+        <v>19259</v>
       </c>
       <c r="N80" t="n">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="O80" t="n">
-        <v>9866</v>
+        <v>9868</v>
       </c>
     </row>
     <row r="81">
@@ -5020,46 +5020,46 @@
         </is>
       </c>
       <c r="C81" t="n">
-        <v>20267</v>
+        <v>37847</v>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/mlf/metalurgia-10000j-50m-1_1000tr-lognormald-20267c_mlf.xlsx</t>
+          <t>Job To Machine/problemset/solution/mlf/metalurgia-10000j-50m-1_1000tr-lognormald-37847.0c_mlf.xlsx</t>
         </is>
       </c>
       <c r="E81" t="n">
-        <v>20266</v>
+        <v>22284</v>
       </c>
       <c r="F81" t="n">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="G81" t="n">
         <v>10000</v>
       </c>
       <c r="H81" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/sjf/metalurgia-10000j-50m-1_1000tr-lognormald-20267c_sjf.xlsx</t>
+          <t>Job To Machine/problemset/solution/sjf/metalurgia-10000j-50m-1_1000tr-lognormald-37847.0c_sjf.xlsx</t>
         </is>
       </c>
       <c r="I81" t="n">
-        <v>20266</v>
+        <v>22284</v>
       </c>
       <c r="J81" t="n">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="K81" t="n">
         <v>10000</v>
       </c>
       <c r="L81" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/ljf/metalurgia-10000j-50m-1_1000tr-lognormald-20267c_ljf.xlsx</t>
+          <t>Job To Machine/problemset/solution/ljf/metalurgia-10000j-50m-1_1000tr-lognormald-37847.0c_ljf.xlsx</t>
         </is>
       </c>
       <c r="M81" t="n">
-        <v>20266</v>
+        <v>22284</v>
       </c>
       <c r="N81" t="n">
-        <v>100</v>
+        <v>96</v>
       </c>
       <c r="O81" t="n">
         <v>10000</v>
@@ -5077,49 +5077,49 @@
         </is>
       </c>
       <c r="C82" t="n">
-        <v>2400</v>
+        <v>1600</v>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/mlf/metalurgia-10000j-50m-1_1000tr-same_per_machined-2400c_mlf.xlsx</t>
+          <t>Job To Machine/problemset/solution/mlf/metalurgia-10000j-50m-1_1000tr-same_per_machined-1600c_mlf.xlsx</t>
         </is>
       </c>
       <c r="E82" t="n">
-        <v>2400</v>
+        <v>1600</v>
       </c>
       <c r="F82" t="n">
         <v>142</v>
       </c>
       <c r="G82" t="n">
-        <v>748</v>
+        <v>470</v>
       </c>
       <c r="H82" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/sjf/metalurgia-10000j-50m-1_1000tr-same_per_machined-2400c_sjf.xlsx</t>
+          <t>Job To Machine/problemset/solution/sjf/metalurgia-10000j-50m-1_1000tr-same_per_machined-1600c_sjf.xlsx</t>
         </is>
       </c>
       <c r="I82" t="n">
-        <v>2400</v>
+        <v>1600</v>
       </c>
       <c r="J82" t="n">
         <v>142</v>
       </c>
       <c r="K82" t="n">
-        <v>748</v>
+        <v>470</v>
       </c>
       <c r="L82" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/ljf/metalurgia-10000j-50m-1_1000tr-same_per_machined-2400c_ljf.xlsx</t>
+          <t>Job To Machine/problemset/solution/ljf/metalurgia-10000j-50m-1_1000tr-same_per_machined-1600c_ljf.xlsx</t>
         </is>
       </c>
       <c r="M82" t="n">
-        <v>2400</v>
+        <v>1600</v>
       </c>
       <c r="N82" t="n">
         <v>142</v>
       </c>
       <c r="O82" t="n">
-        <v>748</v>
+        <v>470</v>
       </c>
     </row>
     <row r="83">
@@ -5134,49 +5134,49 @@
         </is>
       </c>
       <c r="C83" t="n">
-        <v>2448</v>
+        <v>43800</v>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/mlf/metalurgia-10000j-50m-1_1000tr-same_per_machined-2448c_mlf.xlsx</t>
+          <t>Job To Machine/problemset/solution/mlf/metalurgia-10000j-50m-1_1000tr-same_per_machined-43800.0c_mlf.xlsx</t>
         </is>
       </c>
       <c r="E83" t="n">
-        <v>2448</v>
+        <v>43800</v>
       </c>
       <c r="F83" t="n">
-        <v>141</v>
+        <v>46</v>
       </c>
       <c r="G83" t="n">
-        <v>763</v>
+        <v>10000</v>
       </c>
       <c r="H83" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/sjf/metalurgia-10000j-50m-1_1000tr-same_per_machined-2448c_sjf.xlsx</t>
+          <t>Job To Machine/problemset/solution/sjf/metalurgia-10000j-50m-1_1000tr-same_per_machined-43800.0c_sjf.xlsx</t>
         </is>
       </c>
       <c r="I83" t="n">
-        <v>2448</v>
+        <v>43800</v>
       </c>
       <c r="J83" t="n">
-        <v>141</v>
+        <v>46</v>
       </c>
       <c r="K83" t="n">
-        <v>763</v>
+        <v>10000</v>
       </c>
       <c r="L83" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/ljf/metalurgia-10000j-50m-1_1000tr-same_per_machined-2448c_ljf.xlsx</t>
+          <t>Job To Machine/problemset/solution/ljf/metalurgia-10000j-50m-1_1000tr-same_per_machined-43800.0c_ljf.xlsx</t>
         </is>
       </c>
       <c r="M83" t="n">
-        <v>2448</v>
+        <v>43800</v>
       </c>
       <c r="N83" t="n">
-        <v>141</v>
+        <v>46</v>
       </c>
       <c r="O83" t="n">
-        <v>763</v>
+        <v>10000</v>
       </c>
     </row>
     <row r="84">
@@ -5191,49 +5191,49 @@
         </is>
       </c>
       <c r="C84" t="n">
-        <v>98847</v>
+        <v>99936</v>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/mlf/metalurgia-10000j-50m-1_1000tr-same_per_jobd-98847c_mlf.xlsx</t>
+          <t>Job To Machine/problemset/solution/mlf/metalurgia-10000j-50m-1_1000tr-same_per_jobd-99936c_mlf.xlsx</t>
         </is>
       </c>
       <c r="E84" t="n">
-        <v>98847</v>
+        <v>99936</v>
       </c>
       <c r="F84" t="n">
-        <v>494</v>
+        <v>499</v>
       </c>
       <c r="G84" t="n">
         <v>9999</v>
       </c>
       <c r="H84" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/sjf/metalurgia-10000j-50m-1_1000tr-same_per_jobd-98847c_sjf.xlsx</t>
+          <t>Job To Machine/problemset/solution/sjf/metalurgia-10000j-50m-1_1000tr-same_per_jobd-99936c_sjf.xlsx</t>
         </is>
       </c>
       <c r="I84" t="n">
-        <v>98847</v>
+        <v>99924</v>
       </c>
       <c r="J84" t="n">
-        <v>494</v>
+        <v>498</v>
       </c>
       <c r="K84" t="n">
-        <v>9999</v>
+        <v>9982</v>
       </c>
       <c r="L84" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/ljf/metalurgia-10000j-50m-1_1000tr-same_per_jobd-98847c_ljf.xlsx</t>
+          <t>Job To Machine/problemset/solution/ljf/metalurgia-10000j-50m-1_1000tr-same_per_jobd-99936c_ljf.xlsx</t>
         </is>
       </c>
       <c r="M84" t="n">
-        <v>98847</v>
+        <v>99924</v>
       </c>
       <c r="N84" t="n">
-        <v>494</v>
+        <v>498</v>
       </c>
       <c r="O84" t="n">
-        <v>9999</v>
+        <v>9982</v>
       </c>
     </row>
     <row r="85">
@@ -5248,49 +5248,49 @@
         </is>
       </c>
       <c r="C85" t="n">
-        <v>100865</v>
+        <v>99937</v>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/mlf/metalurgia-10000j-50m-1_1000tr-same_per_jobd-100865c_mlf.xlsx</t>
+          <t>Job To Machine/problemset/solution/mlf/metalurgia-10000j-50m-1_1000tr-same_per_jobd-99937.0c_mlf.xlsx</t>
         </is>
       </c>
       <c r="E85" t="n">
-        <v>100865</v>
+        <v>99937</v>
       </c>
       <c r="F85" t="n">
-        <v>494</v>
+        <v>499</v>
       </c>
       <c r="G85" t="n">
-        <v>10000</v>
+        <v>9999</v>
       </c>
       <c r="H85" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/sjf/metalurgia-10000j-50m-1_1000tr-same_per_jobd-100865c_sjf.xlsx</t>
+          <t>Job To Machine/problemset/solution/sjf/metalurgia-10000j-50m-1_1000tr-same_per_jobd-99937.0c_sjf.xlsx</t>
         </is>
       </c>
       <c r="I85" t="n">
-        <v>100865</v>
+        <v>99924</v>
       </c>
       <c r="J85" t="n">
-        <v>494</v>
+        <v>498</v>
       </c>
       <c r="K85" t="n">
-        <v>10000</v>
+        <v>9982</v>
       </c>
       <c r="L85" t="inlineStr">
         <is>
-          <t>Job To Machine/problemset/solution/ljf/metalurgia-10000j-50m-1_1000tr-same_per_jobd-100865c_ljf.xlsx</t>
+          <t>Job To Machine/problemset/solution/ljf/metalurgia-10000j-50m-1_1000tr-same_per_jobd-99937.0c_ljf.xlsx</t>
         </is>
       </c>
       <c r="M85" t="n">
-        <v>100865</v>
+        <v>99924</v>
       </c>
       <c r="N85" t="n">
-        <v>494</v>
+        <v>498</v>
       </c>
       <c r="O85" t="n">
-        <v>10000</v>
+        <v>9982</v>
       </c>
     </row>
   </sheetData>

</xml_diff>